<commit_message>
ci: raise bench-gate threshold to 20%
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/regression.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/regression.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="152">
   <si>
     <t>EMEA</t>
   </si>
@@ -235,12 +235,6 @@
   </si>
   <si>
     <t>agg_median</t>
-  </si>
-  <si>
-    <t>agg_minifs</t>
-  </si>
-  <si>
-    <t>agg_maxifs</t>
   </si>
   <si>
     <t>lk_vlookup</t>
@@ -1099,10 +1093,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:DW11"/>
+  <dimension ref="A1:DU11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:127">
+    <row r="1" spans="1:125">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -1478,14 +1472,8 @@
       <c r="DU1" t="s">
         <v>140</v>
       </c>
-      <c r="DV1" t="s">
-        <v>141</v>
-      </c>
-      <c r="DW1" t="s">
-        <v>142</v>
-      </c>
     </row>
-    <row r="2" spans="1:127">
+    <row r="2" spans="1:125">
       <c r="A2">
         <v>10.0</v>
       </c>
@@ -1502,7 +1490,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G2" s="1">
         <v>45000.0</v>
@@ -1672,319 +1660,311 @@
         <v>0</v>
       </c>
       <c r="AX2">
-        <f>_xlfn.MINIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
+        <f>VLOOKUP(E2,Lookup1!A:C,2,FALSE)</f>
         <v>0</v>
       </c>
       <c r="AY2">
-        <f>_xlfn.MAXIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
-        <v>0</v>
-      </c>
-      <c r="AZ2">
-        <f>VLOOKUP(E2,Lookup1!A:C,2,FALSE)</f>
+        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ2" cm="1">
+        <f t="array" ref="AZ2">_xlfn.XLOOKUP(E2,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
         <v>0</v>
       </c>
       <c r="BA2">
-        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BB2" cm="1">
-        <f t="array" ref="BB2">_xlfn.XLOOKUP(E2,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
+        <f>MATCH(E2,Lookup1!A:A,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BB2">
+        <f>_xlfn.XMATCH(E2,Lookup1!A:A,0)</f>
         <v>0</v>
       </c>
       <c r="BC2">
-        <f>MATCH(E2,Lookup1!A:A,0)</f>
+        <f>INDEX(Lookup1!B:B,MATCH(E2,Lookup1!A:A,0))</f>
         <v>0</v>
       </c>
       <c r="BD2">
-        <f>_xlfn.XMATCH(E2,Lookup1!A:A,0)</f>
+        <f>CHOOSE(2,"alpha","beta","gamma")</f>
         <v>0</v>
       </c>
       <c r="BE2">
-        <f>INDEX(Lookup1!B:B,MATCH(E2,Lookup1!A:A,0))</f>
+        <f>LEFT(F2,3)</f>
         <v>0</v>
       </c>
       <c r="BF2">
-        <f>CHOOSE(2,"alpha","beta","gamma")</f>
+        <f>RIGHT(F2,3)</f>
         <v>0</v>
       </c>
       <c r="BG2">
-        <f>LEFT(F2,3)</f>
+        <f>MID(F2,2,3)</f>
         <v>0</v>
       </c>
       <c r="BH2">
-        <f>RIGHT(F2,3)</f>
+        <f>LEN(F2)</f>
         <v>0</v>
       </c>
       <c r="BI2">
-        <f>MID(F2,2,3)</f>
+        <f>UPPER(F2)</f>
         <v>0</v>
       </c>
       <c r="BJ2">
-        <f>LEN(F2)</f>
+        <f>LOWER(F2)</f>
         <v>0</v>
       </c>
       <c r="BK2">
-        <f>UPPER(F2)</f>
+        <f>PROPER(F2)</f>
         <v>0</v>
       </c>
       <c r="BL2">
-        <f>LOWER(F2)</f>
+        <f>TRIM(F2)</f>
         <v>0</v>
       </c>
       <c r="BM2">
-        <f>PROPER(F2)</f>
+        <f>CLEAN(F2)</f>
         <v>0</v>
       </c>
       <c r="BN2">
-        <f>TRIM(F2)</f>
+        <f>_xlfn.CONCAT(E2,"-",F2)</f>
         <v>0</v>
       </c>
       <c r="BO2">
-        <f>CLEAN(F2)</f>
+        <f>CONCATENATE(E2,"-",F2)</f>
         <v>0</v>
       </c>
       <c r="BP2">
-        <f>_xlfn.CONCAT(E2,"-",F2)</f>
+        <f>_xlfn.TEXTJOIN("-",TRUE,E2,F2)</f>
         <v>0</v>
       </c>
       <c r="BQ2">
-        <f>CONCATENATE(E2,"-",F2)</f>
+        <f>IFERROR(FIND("l",F2),0)</f>
         <v>0</v>
       </c>
       <c r="BR2">
-        <f>_xlfn.TEXTJOIN("-",TRUE,E2,F2)</f>
+        <f>IFERROR(SEARCH("L",F2),0)</f>
         <v>0</v>
       </c>
       <c r="BS2">
-        <f>IFERROR(FIND("l",F2),0)</f>
+        <f>SUBSTITUTE(F2,"o","0")</f>
         <v>0</v>
       </c>
       <c r="BT2">
-        <f>IFERROR(SEARCH("L",F2),0)</f>
+        <f>REPLACE(F2,1,1,"X")</f>
         <v>0</v>
       </c>
       <c r="BU2">
-        <f>SUBSTITUTE(F2,"o","0")</f>
+        <f>TEXT(C2,"0.00")</f>
         <v>0</v>
       </c>
       <c r="BV2">
-        <f>REPLACE(F2,1,1,"X")</f>
+        <f>VALUE("123.45")</f>
         <v>0</v>
       </c>
       <c r="BW2">
-        <f>TEXT(C2,"0.00")</f>
+        <f>EXACT(F2,"hello")</f>
         <v>0</v>
       </c>
       <c r="BX2">
-        <f>VALUE("123.45")</f>
+        <f>ROUND(B2,1)</f>
         <v>0</v>
       </c>
       <c r="BY2">
-        <f>EXACT(F2,"hello")</f>
+        <f>ROUNDUP(B2,0)</f>
         <v>0</v>
       </c>
       <c r="BZ2">
-        <f>ROUND(B2,1)</f>
+        <f>ROUNDDOWN(B2,0)</f>
         <v>0</v>
       </c>
       <c r="CA2">
-        <f>ROUNDUP(B2,0)</f>
+        <f>INT(B2)</f>
         <v>0</v>
       </c>
       <c r="CB2">
-        <f>ROUNDDOWN(B2,0)</f>
+        <f>MOD(A2,3)</f>
         <v>0</v>
       </c>
       <c r="CC2">
-        <f>INT(B2)</f>
+        <f>ABS(A2)</f>
         <v>0</v>
       </c>
       <c r="CD2">
-        <f>MOD(A2,3)</f>
+        <f>SIGN(A2)</f>
         <v>0</v>
       </c>
       <c r="CE2">
-        <f>ABS(A2)</f>
+        <f>SQRT(ABS(A2))</f>
         <v>0</v>
       </c>
       <c r="CF2">
-        <f>SIGN(A2)</f>
+        <f>POWER(ABS(A2),2)</f>
         <v>0</v>
       </c>
       <c r="CG2">
-        <f>SQRT(ABS(A2))</f>
+        <f>CEILING(B2,1)</f>
         <v>0</v>
       </c>
       <c r="CH2">
-        <f>POWER(ABS(A2),2)</f>
+        <f>FLOOR(B2,1)</f>
         <v>0</v>
       </c>
       <c r="CI2">
-        <f>CEILING(B2,1)</f>
+        <f>LN(ABS(A2)+1)</f>
         <v>0</v>
       </c>
       <c r="CJ2">
-        <f>FLOOR(B2,1)</f>
+        <f>LOG(ABS(A2)+1,10)</f>
         <v>0</v>
       </c>
       <c r="CK2">
-        <f>LN(ABS(A2)+1)</f>
+        <f>LOG10(ABS(A2)+1)</f>
         <v>0</v>
       </c>
       <c r="CL2">
-        <f>LOG(ABS(A2)+1,10)</f>
+        <f>EXP(1)</f>
         <v>0</v>
       </c>
       <c r="CM2">
-        <f>LOG10(ABS(A2)+1)</f>
+        <f>SIN(B2)</f>
         <v>0</v>
       </c>
       <c r="CN2">
-        <f>EXP(1)</f>
+        <f>COS(B2)</f>
         <v>0</v>
       </c>
       <c r="CO2">
-        <f>SIN(B2)</f>
+        <f>TAN(B2)</f>
         <v>0</v>
       </c>
       <c r="CP2">
-        <f>COS(B2)</f>
+        <f>ASIN(B2/100)</f>
         <v>0</v>
       </c>
       <c r="CQ2">
-        <f>TAN(B2)</f>
+        <f>ACOS(B2/100)</f>
         <v>0</v>
       </c>
       <c r="CR2">
-        <f>ASIN(B2/100)</f>
+        <f>ATAN(B2)</f>
         <v>0</v>
       </c>
       <c r="CS2">
-        <f>ACOS(B2/100)</f>
+        <f>ATAN2(A2,B2)</f>
         <v>0</v>
       </c>
       <c r="CT2">
-        <f>ATAN(B2)</f>
+        <f>PI()</f>
         <v>0</v>
       </c>
       <c r="CU2">
-        <f>ATAN2(A2,B2)</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
       <c r="CV2">
-        <f>PI()</f>
+        <f>NOW()</f>
         <v>0</v>
       </c>
       <c r="CW2">
-        <f>TODAY()</f>
+        <f>DATE(2026,4,20)</f>
         <v>0</v>
       </c>
       <c r="CX2">
-        <f>NOW()</f>
+        <f>YEAR(G2)</f>
         <v>0</v>
       </c>
       <c r="CY2">
-        <f>DATE(2026,4,20)</f>
+        <f>MONTH(G2)</f>
         <v>0</v>
       </c>
       <c r="CZ2">
-        <f>YEAR(G2)</f>
+        <f>DAY(G2)</f>
         <v>0</v>
       </c>
       <c r="DA2">
-        <f>MONTH(G2)</f>
+        <f>WEEKDAY(G2)</f>
         <v>0</v>
       </c>
       <c r="DB2">
-        <f>DAY(G2)</f>
+        <f>EDATE(G2,3)</f>
         <v>0</v>
       </c>
       <c r="DC2">
-        <f>WEEKDAY(G2)</f>
+        <f>EOMONTH(G2,0)</f>
         <v>0</v>
       </c>
       <c r="DD2">
-        <f>EDATE(G2,3)</f>
+        <f>DATEDIF(DATE(2020,1,1),G2,"d")</f>
         <v>0</v>
       </c>
       <c r="DE2">
-        <f>EOMONTH(G2,0)</f>
+        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
         <v>0</v>
       </c>
       <c r="DF2">
-        <f>DATEDIF(DATE(2020,1,1),G2,"d")</f>
+        <f>WORKDAY(DATE(2026,1,1),10)</f>
         <v>0</v>
       </c>
       <c r="DG2">
-        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
+        <f>ISBLANK(H2)</f>
         <v>0</v>
       </c>
       <c r="DH2">
-        <f>WORKDAY(DATE(2026,1,1),10)</f>
+        <f>ISNUMBER(A2)</f>
         <v>0</v>
       </c>
       <c r="DI2">
-        <f>ISBLANK(H2)</f>
+        <f>ISTEXT(F2)</f>
         <v>0</v>
       </c>
       <c r="DJ2">
-        <f>ISNUMBER(A2)</f>
+        <f>ISLOGICAL(D2)</f>
         <v>0</v>
       </c>
       <c r="DK2">
-        <f>ISTEXT(F2)</f>
+        <f>ISNONTEXT(A2)</f>
         <v>0</v>
       </c>
       <c r="DL2">
-        <f>ISLOGICAL(D2)</f>
+        <f>ISERROR(1/0)</f>
         <v>0</v>
       </c>
       <c r="DM2">
-        <f>ISNONTEXT(A2)</f>
+        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="DN2">
-        <f>ISERROR(1/0)</f>
+        <f>ISREF(A2)</f>
         <v>0</v>
       </c>
       <c r="DO2">
-        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
+        <f>NA()</f>
         <v>0</v>
       </c>
       <c r="DP2">
-        <f>ISREF(A2)</f>
+        <f>TYPE(A2)</f>
         <v>0</v>
       </c>
       <c r="DQ2">
-        <f>NA()</f>
+        <f>PMT(0.05/12,360,-200000)</f>
         <v>0</v>
       </c>
       <c r="DR2">
-        <f>TYPE(A2)</f>
+        <f>PV(0.08/12,120,-500)</f>
         <v>0</v>
       </c>
       <c r="DS2">
-        <f>PMT(0.05/12,360,-200000)</f>
+        <f>FV(0.06/12,240,-200)</f>
         <v>0</v>
       </c>
       <c r="DT2">
-        <f>PV(0.08/12,120,-500)</f>
+        <f>NPV(0.1,A2,B2,C2)</f>
         <v>0</v>
       </c>
       <c r="DU2">
-        <f>FV(0.06/12,240,-200)</f>
-        <v>0</v>
-      </c>
-      <c r="DV2">
-        <f>NPV(0.1,A2,B2,C2)</f>
-        <v>0</v>
-      </c>
-      <c r="DW2">
         <f>RATE(120,-500,50000)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:127">
+    <row r="3" spans="1:125">
       <c r="A3">
         <v>25.0</v>
       </c>
@@ -2001,7 +1981,7 @@
         <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G3" s="1">
         <v>45031.0</v>
@@ -2174,319 +2154,311 @@
         <v>0</v>
       </c>
       <c r="AX3">
-        <f>_xlfn.MINIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
+        <f>VLOOKUP(E3,Lookup1!A:C,2,FALSE)</f>
         <v>0</v>
       </c>
       <c r="AY3">
-        <f>_xlfn.MAXIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
-        <v>0</v>
-      </c>
-      <c r="AZ3">
-        <f>VLOOKUP(E3,Lookup1!A:C,2,FALSE)</f>
+        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ3" cm="1">
+        <f t="array" ref="AZ3">_xlfn.XLOOKUP(E3,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
         <v>0</v>
       </c>
       <c r="BA3">
-        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BB3" cm="1">
-        <f t="array" ref="BB3">_xlfn.XLOOKUP(E3,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
+        <f>MATCH(E3,Lookup1!A:A,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BB3">
+        <f>_xlfn.XMATCH(E3,Lookup1!A:A,0)</f>
         <v>0</v>
       </c>
       <c r="BC3">
-        <f>MATCH(E3,Lookup1!A:A,0)</f>
+        <f>INDEX(Lookup1!B:B,MATCH(E3,Lookup1!A:A,0))</f>
         <v>0</v>
       </c>
       <c r="BD3">
-        <f>_xlfn.XMATCH(E3,Lookup1!A:A,0)</f>
+        <f>CHOOSE(2,"alpha","beta","gamma")</f>
         <v>0</v>
       </c>
       <c r="BE3">
-        <f>INDEX(Lookup1!B:B,MATCH(E3,Lookup1!A:A,0))</f>
+        <f>LEFT(F3,3)</f>
         <v>0</v>
       </c>
       <c r="BF3">
-        <f>CHOOSE(2,"alpha","beta","gamma")</f>
+        <f>RIGHT(F3,3)</f>
         <v>0</v>
       </c>
       <c r="BG3">
-        <f>LEFT(F3,3)</f>
+        <f>MID(F3,2,3)</f>
         <v>0</v>
       </c>
       <c r="BH3">
-        <f>RIGHT(F3,3)</f>
+        <f>LEN(F3)</f>
         <v>0</v>
       </c>
       <c r="BI3">
-        <f>MID(F3,2,3)</f>
+        <f>UPPER(F3)</f>
         <v>0</v>
       </c>
       <c r="BJ3">
-        <f>LEN(F3)</f>
+        <f>LOWER(F3)</f>
         <v>0</v>
       </c>
       <c r="BK3">
-        <f>UPPER(F3)</f>
+        <f>PROPER(F3)</f>
         <v>0</v>
       </c>
       <c r="BL3">
-        <f>LOWER(F3)</f>
+        <f>TRIM(F3)</f>
         <v>0</v>
       </c>
       <c r="BM3">
-        <f>PROPER(F3)</f>
+        <f>CLEAN(F3)</f>
         <v>0</v>
       </c>
       <c r="BN3">
-        <f>TRIM(F3)</f>
+        <f>_xlfn.CONCAT(E3,"-",F3)</f>
         <v>0</v>
       </c>
       <c r="BO3">
-        <f>CLEAN(F3)</f>
+        <f>CONCATENATE(E3,"-",F3)</f>
         <v>0</v>
       </c>
       <c r="BP3">
-        <f>_xlfn.CONCAT(E3,"-",F3)</f>
+        <f>_xlfn.TEXTJOIN("-",TRUE,E3,F3)</f>
         <v>0</v>
       </c>
       <c r="BQ3">
-        <f>CONCATENATE(E3,"-",F3)</f>
+        <f>IFERROR(FIND("l",F3),0)</f>
         <v>0</v>
       </c>
       <c r="BR3">
-        <f>_xlfn.TEXTJOIN("-",TRUE,E3,F3)</f>
+        <f>IFERROR(SEARCH("L",F3),0)</f>
         <v>0</v>
       </c>
       <c r="BS3">
-        <f>IFERROR(FIND("l",F3),0)</f>
+        <f>SUBSTITUTE(F3,"o","0")</f>
         <v>0</v>
       </c>
       <c r="BT3">
-        <f>IFERROR(SEARCH("L",F3),0)</f>
+        <f>REPLACE(F3,1,1,"X")</f>
         <v>0</v>
       </c>
       <c r="BU3">
-        <f>SUBSTITUTE(F3,"o","0")</f>
+        <f>TEXT(C3,"0.00")</f>
         <v>0</v>
       </c>
       <c r="BV3">
-        <f>REPLACE(F3,1,1,"X")</f>
+        <f>VALUE("123.45")</f>
         <v>0</v>
       </c>
       <c r="BW3">
-        <f>TEXT(C3,"0.00")</f>
+        <f>EXACT(F3,"hello")</f>
         <v>0</v>
       </c>
       <c r="BX3">
-        <f>VALUE("123.45")</f>
+        <f>ROUND(B3,1)</f>
         <v>0</v>
       </c>
       <c r="BY3">
-        <f>EXACT(F3,"hello")</f>
+        <f>ROUNDUP(B3,0)</f>
         <v>0</v>
       </c>
       <c r="BZ3">
-        <f>ROUND(B3,1)</f>
+        <f>ROUNDDOWN(B3,0)</f>
         <v>0</v>
       </c>
       <c r="CA3">
-        <f>ROUNDUP(B3,0)</f>
+        <f>INT(B3)</f>
         <v>0</v>
       </c>
       <c r="CB3">
-        <f>ROUNDDOWN(B3,0)</f>
+        <f>MOD(A3,3)</f>
         <v>0</v>
       </c>
       <c r="CC3">
-        <f>INT(B3)</f>
+        <f>ABS(A3)</f>
         <v>0</v>
       </c>
       <c r="CD3">
-        <f>MOD(A3,3)</f>
+        <f>SIGN(A3)</f>
         <v>0</v>
       </c>
       <c r="CE3">
-        <f>ABS(A3)</f>
+        <f>SQRT(ABS(A3))</f>
         <v>0</v>
       </c>
       <c r="CF3">
-        <f>SIGN(A3)</f>
+        <f>POWER(ABS(A3),2)</f>
         <v>0</v>
       </c>
       <c r="CG3">
-        <f>SQRT(ABS(A3))</f>
+        <f>CEILING(B3,1)</f>
         <v>0</v>
       </c>
       <c r="CH3">
-        <f>POWER(ABS(A3),2)</f>
+        <f>FLOOR(B3,1)</f>
         <v>0</v>
       </c>
       <c r="CI3">
-        <f>CEILING(B3,1)</f>
+        <f>LN(ABS(A3)+1)</f>
         <v>0</v>
       </c>
       <c r="CJ3">
-        <f>FLOOR(B3,1)</f>
+        <f>LOG(ABS(A3)+1,10)</f>
         <v>0</v>
       </c>
       <c r="CK3">
-        <f>LN(ABS(A3)+1)</f>
+        <f>LOG10(ABS(A3)+1)</f>
         <v>0</v>
       </c>
       <c r="CL3">
-        <f>LOG(ABS(A3)+1,10)</f>
+        <f>EXP(1)</f>
         <v>0</v>
       </c>
       <c r="CM3">
-        <f>LOG10(ABS(A3)+1)</f>
+        <f>SIN(B3)</f>
         <v>0</v>
       </c>
       <c r="CN3">
-        <f>EXP(1)</f>
+        <f>COS(B3)</f>
         <v>0</v>
       </c>
       <c r="CO3">
-        <f>SIN(B3)</f>
+        <f>TAN(B3)</f>
         <v>0</v>
       </c>
       <c r="CP3">
-        <f>COS(B3)</f>
+        <f>ASIN(B3/100)</f>
         <v>0</v>
       </c>
       <c r="CQ3">
-        <f>TAN(B3)</f>
+        <f>ACOS(B3/100)</f>
         <v>0</v>
       </c>
       <c r="CR3">
-        <f>ASIN(B3/100)</f>
+        <f>ATAN(B3)</f>
         <v>0</v>
       </c>
       <c r="CS3">
-        <f>ACOS(B3/100)</f>
+        <f>ATAN2(A3,B3)</f>
         <v>0</v>
       </c>
       <c r="CT3">
-        <f>ATAN(B3)</f>
+        <f>PI()</f>
         <v>0</v>
       </c>
       <c r="CU3">
-        <f>ATAN2(A3,B3)</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
       <c r="CV3">
-        <f>PI()</f>
+        <f>NOW()</f>
         <v>0</v>
       </c>
       <c r="CW3">
-        <f>TODAY()</f>
+        <f>DATE(2026,4,20)</f>
         <v>0</v>
       </c>
       <c r="CX3">
-        <f>NOW()</f>
+        <f>YEAR(G3)</f>
         <v>0</v>
       </c>
       <c r="CY3">
-        <f>DATE(2026,4,20)</f>
+        <f>MONTH(G3)</f>
         <v>0</v>
       </c>
       <c r="CZ3">
-        <f>YEAR(G3)</f>
+        <f>DAY(G3)</f>
         <v>0</v>
       </c>
       <c r="DA3">
-        <f>MONTH(G3)</f>
+        <f>WEEKDAY(G3)</f>
         <v>0</v>
       </c>
       <c r="DB3">
-        <f>DAY(G3)</f>
+        <f>EDATE(G3,3)</f>
         <v>0</v>
       </c>
       <c r="DC3">
-        <f>WEEKDAY(G3)</f>
+        <f>EOMONTH(G3,0)</f>
         <v>0</v>
       </c>
       <c r="DD3">
-        <f>EDATE(G3,3)</f>
+        <f>DATEDIF(DATE(2020,1,1),G3,"d")</f>
         <v>0</v>
       </c>
       <c r="DE3">
-        <f>EOMONTH(G3,0)</f>
+        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
         <v>0</v>
       </c>
       <c r="DF3">
-        <f>DATEDIF(DATE(2020,1,1),G3,"d")</f>
+        <f>WORKDAY(DATE(2026,1,1),10)</f>
         <v>0</v>
       </c>
       <c r="DG3">
-        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
+        <f>ISBLANK(H3)</f>
         <v>0</v>
       </c>
       <c r="DH3">
-        <f>WORKDAY(DATE(2026,1,1),10)</f>
+        <f>ISNUMBER(A3)</f>
         <v>0</v>
       </c>
       <c r="DI3">
-        <f>ISBLANK(H3)</f>
+        <f>ISTEXT(F3)</f>
         <v>0</v>
       </c>
       <c r="DJ3">
-        <f>ISNUMBER(A3)</f>
+        <f>ISLOGICAL(D3)</f>
         <v>0</v>
       </c>
       <c r="DK3">
-        <f>ISTEXT(F3)</f>
+        <f>ISNONTEXT(A3)</f>
         <v>0</v>
       </c>
       <c r="DL3">
-        <f>ISLOGICAL(D3)</f>
+        <f>ISERROR(1/0)</f>
         <v>0</v>
       </c>
       <c r="DM3">
-        <f>ISNONTEXT(A3)</f>
+        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="DN3">
-        <f>ISERROR(1/0)</f>
+        <f>ISREF(A3)</f>
         <v>0</v>
       </c>
       <c r="DO3">
-        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
+        <f>NA()</f>
         <v>0</v>
       </c>
       <c r="DP3">
-        <f>ISREF(A3)</f>
+        <f>TYPE(A3)</f>
         <v>0</v>
       </c>
       <c r="DQ3">
-        <f>NA()</f>
+        <f>PMT(0.05/12,360,-200000)</f>
         <v>0</v>
       </c>
       <c r="DR3">
-        <f>TYPE(A3)</f>
+        <f>PV(0.08/12,120,-500)</f>
         <v>0</v>
       </c>
       <c r="DS3">
-        <f>PMT(0.05/12,360,-200000)</f>
+        <f>FV(0.06/12,240,-200)</f>
         <v>0</v>
       </c>
       <c r="DT3">
-        <f>PV(0.08/12,120,-500)</f>
+        <f>NPV(0.1,A3,B3,C3)</f>
         <v>0</v>
       </c>
       <c r="DU3">
-        <f>FV(0.06/12,240,-200)</f>
-        <v>0</v>
-      </c>
-      <c r="DV3">
-        <f>NPV(0.1,A3,B3,C3)</f>
-        <v>0</v>
-      </c>
-      <c r="DW3">
         <f>RATE(120,-500,50000)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:127">
+    <row r="4" spans="1:125">
       <c r="A4">
         <v>0.0</v>
       </c>
@@ -2503,7 +2475,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G4" s="1">
         <v>45061.0</v>
@@ -2676,319 +2648,311 @@
         <v>0</v>
       </c>
       <c r="AX4">
-        <f>_xlfn.MINIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
+        <f>VLOOKUP(E4,Lookup1!A:C,2,FALSE)</f>
         <v>0</v>
       </c>
       <c r="AY4">
-        <f>_xlfn.MAXIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
-        <v>0</v>
-      </c>
-      <c r="AZ4">
-        <f>VLOOKUP(E4,Lookup1!A:C,2,FALSE)</f>
+        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ4" cm="1">
+        <f t="array" ref="AZ4">_xlfn.XLOOKUP(E4,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
         <v>0</v>
       </c>
       <c r="BA4">
-        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BB4" cm="1">
-        <f t="array" ref="BB4">_xlfn.XLOOKUP(E4,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
+        <f>MATCH(E4,Lookup1!A:A,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BB4">
+        <f>_xlfn.XMATCH(E4,Lookup1!A:A,0)</f>
         <v>0</v>
       </c>
       <c r="BC4">
-        <f>MATCH(E4,Lookup1!A:A,0)</f>
+        <f>INDEX(Lookup1!B:B,MATCH(E4,Lookup1!A:A,0))</f>
         <v>0</v>
       </c>
       <c r="BD4">
-        <f>_xlfn.XMATCH(E4,Lookup1!A:A,0)</f>
+        <f>CHOOSE(2,"alpha","beta","gamma")</f>
         <v>0</v>
       </c>
       <c r="BE4">
-        <f>INDEX(Lookup1!B:B,MATCH(E4,Lookup1!A:A,0))</f>
+        <f>LEFT(F4,3)</f>
         <v>0</v>
       </c>
       <c r="BF4">
-        <f>CHOOSE(2,"alpha","beta","gamma")</f>
+        <f>RIGHT(F4,3)</f>
         <v>0</v>
       </c>
       <c r="BG4">
-        <f>LEFT(F4,3)</f>
+        <f>MID(F4,2,3)</f>
         <v>0</v>
       </c>
       <c r="BH4">
-        <f>RIGHT(F4,3)</f>
+        <f>LEN(F4)</f>
         <v>0</v>
       </c>
       <c r="BI4">
-        <f>MID(F4,2,3)</f>
+        <f>UPPER(F4)</f>
         <v>0</v>
       </c>
       <c r="BJ4">
-        <f>LEN(F4)</f>
+        <f>LOWER(F4)</f>
         <v>0</v>
       </c>
       <c r="BK4">
-        <f>UPPER(F4)</f>
+        <f>PROPER(F4)</f>
         <v>0</v>
       </c>
       <c r="BL4">
-        <f>LOWER(F4)</f>
+        <f>TRIM(F4)</f>
         <v>0</v>
       </c>
       <c r="BM4">
-        <f>PROPER(F4)</f>
+        <f>CLEAN(F4)</f>
         <v>0</v>
       </c>
       <c r="BN4">
-        <f>TRIM(F4)</f>
+        <f>_xlfn.CONCAT(E4,"-",F4)</f>
         <v>0</v>
       </c>
       <c r="BO4">
-        <f>CLEAN(F4)</f>
+        <f>CONCATENATE(E4,"-",F4)</f>
         <v>0</v>
       </c>
       <c r="BP4">
-        <f>_xlfn.CONCAT(E4,"-",F4)</f>
+        <f>_xlfn.TEXTJOIN("-",TRUE,E4,F4)</f>
         <v>0</v>
       </c>
       <c r="BQ4">
-        <f>CONCATENATE(E4,"-",F4)</f>
+        <f>IFERROR(FIND("l",F4),0)</f>
         <v>0</v>
       </c>
       <c r="BR4">
-        <f>_xlfn.TEXTJOIN("-",TRUE,E4,F4)</f>
+        <f>IFERROR(SEARCH("L",F4),0)</f>
         <v>0</v>
       </c>
       <c r="BS4">
-        <f>IFERROR(FIND("l",F4),0)</f>
+        <f>SUBSTITUTE(F4,"o","0")</f>
         <v>0</v>
       </c>
       <c r="BT4">
-        <f>IFERROR(SEARCH("L",F4),0)</f>
+        <f>REPLACE(F4,1,1,"X")</f>
         <v>0</v>
       </c>
       <c r="BU4">
-        <f>SUBSTITUTE(F4,"o","0")</f>
+        <f>TEXT(C4,"0.00")</f>
         <v>0</v>
       </c>
       <c r="BV4">
-        <f>REPLACE(F4,1,1,"X")</f>
+        <f>VALUE("123.45")</f>
         <v>0</v>
       </c>
       <c r="BW4">
-        <f>TEXT(C4,"0.00")</f>
+        <f>EXACT(F4,"hello")</f>
         <v>0</v>
       </c>
       <c r="BX4">
-        <f>VALUE("123.45")</f>
+        <f>ROUND(B4,1)</f>
         <v>0</v>
       </c>
       <c r="BY4">
-        <f>EXACT(F4,"hello")</f>
+        <f>ROUNDUP(B4,0)</f>
         <v>0</v>
       </c>
       <c r="BZ4">
-        <f>ROUND(B4,1)</f>
+        <f>ROUNDDOWN(B4,0)</f>
         <v>0</v>
       </c>
       <c r="CA4">
-        <f>ROUNDUP(B4,0)</f>
+        <f>INT(B4)</f>
         <v>0</v>
       </c>
       <c r="CB4">
-        <f>ROUNDDOWN(B4,0)</f>
+        <f>MOD(A4,3)</f>
         <v>0</v>
       </c>
       <c r="CC4">
-        <f>INT(B4)</f>
+        <f>ABS(A4)</f>
         <v>0</v>
       </c>
       <c r="CD4">
-        <f>MOD(A4,3)</f>
+        <f>SIGN(A4)</f>
         <v>0</v>
       </c>
       <c r="CE4">
-        <f>ABS(A4)</f>
+        <f>SQRT(ABS(A4))</f>
         <v>0</v>
       </c>
       <c r="CF4">
-        <f>SIGN(A4)</f>
+        <f>POWER(ABS(A4),2)</f>
         <v>0</v>
       </c>
       <c r="CG4">
-        <f>SQRT(ABS(A4))</f>
+        <f>CEILING(B4,1)</f>
         <v>0</v>
       </c>
       <c r="CH4">
-        <f>POWER(ABS(A4),2)</f>
+        <f>FLOOR(B4,1)</f>
         <v>0</v>
       </c>
       <c r="CI4">
-        <f>CEILING(B4,1)</f>
+        <f>LN(ABS(A4)+1)</f>
         <v>0</v>
       </c>
       <c r="CJ4">
-        <f>FLOOR(B4,1)</f>
+        <f>LOG(ABS(A4)+1,10)</f>
         <v>0</v>
       </c>
       <c r="CK4">
-        <f>LN(ABS(A4)+1)</f>
+        <f>LOG10(ABS(A4)+1)</f>
         <v>0</v>
       </c>
       <c r="CL4">
-        <f>LOG(ABS(A4)+1,10)</f>
+        <f>EXP(1)</f>
         <v>0</v>
       </c>
       <c r="CM4">
-        <f>LOG10(ABS(A4)+1)</f>
+        <f>SIN(B4)</f>
         <v>0</v>
       </c>
       <c r="CN4">
-        <f>EXP(1)</f>
+        <f>COS(B4)</f>
         <v>0</v>
       </c>
       <c r="CO4">
-        <f>SIN(B4)</f>
+        <f>TAN(B4)</f>
         <v>0</v>
       </c>
       <c r="CP4">
-        <f>COS(B4)</f>
+        <f>ASIN(B4/100)</f>
         <v>0</v>
       </c>
       <c r="CQ4">
-        <f>TAN(B4)</f>
+        <f>ACOS(B4/100)</f>
         <v>0</v>
       </c>
       <c r="CR4">
-        <f>ASIN(B4/100)</f>
+        <f>ATAN(B4)</f>
         <v>0</v>
       </c>
       <c r="CS4">
-        <f>ACOS(B4/100)</f>
+        <f>ATAN2(A4,B4)</f>
         <v>0</v>
       </c>
       <c r="CT4">
-        <f>ATAN(B4)</f>
+        <f>PI()</f>
         <v>0</v>
       </c>
       <c r="CU4">
-        <f>ATAN2(A4,B4)</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
       <c r="CV4">
-        <f>PI()</f>
+        <f>NOW()</f>
         <v>0</v>
       </c>
       <c r="CW4">
-        <f>TODAY()</f>
+        <f>DATE(2026,4,20)</f>
         <v>0</v>
       </c>
       <c r="CX4">
-        <f>NOW()</f>
+        <f>YEAR(G4)</f>
         <v>0</v>
       </c>
       <c r="CY4">
-        <f>DATE(2026,4,20)</f>
+        <f>MONTH(G4)</f>
         <v>0</v>
       </c>
       <c r="CZ4">
-        <f>YEAR(G4)</f>
+        <f>DAY(G4)</f>
         <v>0</v>
       </c>
       <c r="DA4">
-        <f>MONTH(G4)</f>
+        <f>WEEKDAY(G4)</f>
         <v>0</v>
       </c>
       <c r="DB4">
-        <f>DAY(G4)</f>
+        <f>EDATE(G4,3)</f>
         <v>0</v>
       </c>
       <c r="DC4">
-        <f>WEEKDAY(G4)</f>
+        <f>EOMONTH(G4,0)</f>
         <v>0</v>
       </c>
       <c r="DD4">
-        <f>EDATE(G4,3)</f>
+        <f>DATEDIF(DATE(2020,1,1),G4,"d")</f>
         <v>0</v>
       </c>
       <c r="DE4">
-        <f>EOMONTH(G4,0)</f>
+        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
         <v>0</v>
       </c>
       <c r="DF4">
-        <f>DATEDIF(DATE(2020,1,1),G4,"d")</f>
+        <f>WORKDAY(DATE(2026,1,1),10)</f>
         <v>0</v>
       </c>
       <c r="DG4">
-        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
+        <f>ISBLANK(H4)</f>
         <v>0</v>
       </c>
       <c r="DH4">
-        <f>WORKDAY(DATE(2026,1,1),10)</f>
+        <f>ISNUMBER(A4)</f>
         <v>0</v>
       </c>
       <c r="DI4">
-        <f>ISBLANK(H4)</f>
+        <f>ISTEXT(F4)</f>
         <v>0</v>
       </c>
       <c r="DJ4">
-        <f>ISNUMBER(A4)</f>
+        <f>ISLOGICAL(D4)</f>
         <v>0</v>
       </c>
       <c r="DK4">
-        <f>ISTEXT(F4)</f>
+        <f>ISNONTEXT(A4)</f>
         <v>0</v>
       </c>
       <c r="DL4">
-        <f>ISLOGICAL(D4)</f>
+        <f>ISERROR(1/0)</f>
         <v>0</v>
       </c>
       <c r="DM4">
-        <f>ISNONTEXT(A4)</f>
+        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="DN4">
-        <f>ISERROR(1/0)</f>
+        <f>ISREF(A4)</f>
         <v>0</v>
       </c>
       <c r="DO4">
-        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
+        <f>NA()</f>
         <v>0</v>
       </c>
       <c r="DP4">
-        <f>ISREF(A4)</f>
+        <f>TYPE(A4)</f>
         <v>0</v>
       </c>
       <c r="DQ4">
-        <f>NA()</f>
+        <f>PMT(0.05/12,360,-200000)</f>
         <v>0</v>
       </c>
       <c r="DR4">
-        <f>TYPE(A4)</f>
+        <f>PV(0.08/12,120,-500)</f>
         <v>0</v>
       </c>
       <c r="DS4">
-        <f>PMT(0.05/12,360,-200000)</f>
+        <f>FV(0.06/12,240,-200)</f>
         <v>0</v>
       </c>
       <c r="DT4">
-        <f>PV(0.08/12,120,-500)</f>
+        <f>NPV(0.1,A4,B4,C4)</f>
         <v>0</v>
       </c>
       <c r="DU4">
-        <f>FV(0.06/12,240,-200)</f>
-        <v>0</v>
-      </c>
-      <c r="DV4">
-        <f>NPV(0.1,A4,B4,C4)</f>
-        <v>0</v>
-      </c>
-      <c r="DW4">
         <f>RATE(120,-500,50000)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:127">
+    <row r="5" spans="1:125">
       <c r="A5">
         <v>100.0</v>
       </c>
@@ -3005,7 +2969,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G5" s="1">
         <v>44927.0</v>
@@ -3175,319 +3139,311 @@
         <v>0</v>
       </c>
       <c r="AX5">
-        <f>_xlfn.MINIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
+        <f>VLOOKUP(E5,Lookup1!A:C,2,FALSE)</f>
         <v>0</v>
       </c>
       <c r="AY5">
-        <f>_xlfn.MAXIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
-        <v>0</v>
-      </c>
-      <c r="AZ5">
-        <f>VLOOKUP(E5,Lookup1!A:C,2,FALSE)</f>
+        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ5" cm="1">
+        <f t="array" ref="AZ5">_xlfn.XLOOKUP(E5,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
         <v>0</v>
       </c>
       <c r="BA5">
-        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BB5" cm="1">
-        <f t="array" ref="BB5">_xlfn.XLOOKUP(E5,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
+        <f>MATCH(E5,Lookup1!A:A,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BB5">
+        <f>_xlfn.XMATCH(E5,Lookup1!A:A,0)</f>
         <v>0</v>
       </c>
       <c r="BC5">
-        <f>MATCH(E5,Lookup1!A:A,0)</f>
+        <f>INDEX(Lookup1!B:B,MATCH(E5,Lookup1!A:A,0))</f>
         <v>0</v>
       </c>
       <c r="BD5">
-        <f>_xlfn.XMATCH(E5,Lookup1!A:A,0)</f>
+        <f>CHOOSE(2,"alpha","beta","gamma")</f>
         <v>0</v>
       </c>
       <c r="BE5">
-        <f>INDEX(Lookup1!B:B,MATCH(E5,Lookup1!A:A,0))</f>
+        <f>LEFT(F5,3)</f>
         <v>0</v>
       </c>
       <c r="BF5">
-        <f>CHOOSE(2,"alpha","beta","gamma")</f>
+        <f>RIGHT(F5,3)</f>
         <v>0</v>
       </c>
       <c r="BG5">
-        <f>LEFT(F5,3)</f>
+        <f>MID(F5,2,3)</f>
         <v>0</v>
       </c>
       <c r="BH5">
-        <f>RIGHT(F5,3)</f>
+        <f>LEN(F5)</f>
         <v>0</v>
       </c>
       <c r="BI5">
-        <f>MID(F5,2,3)</f>
+        <f>UPPER(F5)</f>
         <v>0</v>
       </c>
       <c r="BJ5">
-        <f>LEN(F5)</f>
+        <f>LOWER(F5)</f>
         <v>0</v>
       </c>
       <c r="BK5">
-        <f>UPPER(F5)</f>
+        <f>PROPER(F5)</f>
         <v>0</v>
       </c>
       <c r="BL5">
-        <f>LOWER(F5)</f>
+        <f>TRIM(F5)</f>
         <v>0</v>
       </c>
       <c r="BM5">
-        <f>PROPER(F5)</f>
+        <f>CLEAN(F5)</f>
         <v>0</v>
       </c>
       <c r="BN5">
-        <f>TRIM(F5)</f>
+        <f>_xlfn.CONCAT(E5,"-",F5)</f>
         <v>0</v>
       </c>
       <c r="BO5">
-        <f>CLEAN(F5)</f>
+        <f>CONCATENATE(E5,"-",F5)</f>
         <v>0</v>
       </c>
       <c r="BP5">
-        <f>_xlfn.CONCAT(E5,"-",F5)</f>
+        <f>_xlfn.TEXTJOIN("-",TRUE,E5,F5)</f>
         <v>0</v>
       </c>
       <c r="BQ5">
-        <f>CONCATENATE(E5,"-",F5)</f>
+        <f>IFERROR(FIND("l",F5),0)</f>
         <v>0</v>
       </c>
       <c r="BR5">
-        <f>_xlfn.TEXTJOIN("-",TRUE,E5,F5)</f>
+        <f>IFERROR(SEARCH("L",F5),0)</f>
         <v>0</v>
       </c>
       <c r="BS5">
-        <f>IFERROR(FIND("l",F5),0)</f>
+        <f>SUBSTITUTE(F5,"o","0")</f>
         <v>0</v>
       </c>
       <c r="BT5">
-        <f>IFERROR(SEARCH("L",F5),0)</f>
+        <f>REPLACE(F5,1,1,"X")</f>
         <v>0</v>
       </c>
       <c r="BU5">
-        <f>SUBSTITUTE(F5,"o","0")</f>
+        <f>TEXT(C5,"0.00")</f>
         <v>0</v>
       </c>
       <c r="BV5">
-        <f>REPLACE(F5,1,1,"X")</f>
+        <f>VALUE("123.45")</f>
         <v>0</v>
       </c>
       <c r="BW5">
-        <f>TEXT(C5,"0.00")</f>
+        <f>EXACT(F5,"hello")</f>
         <v>0</v>
       </c>
       <c r="BX5">
-        <f>VALUE("123.45")</f>
+        <f>ROUND(B5,1)</f>
         <v>0</v>
       </c>
       <c r="BY5">
-        <f>EXACT(F5,"hello")</f>
+        <f>ROUNDUP(B5,0)</f>
         <v>0</v>
       </c>
       <c r="BZ5">
-        <f>ROUND(B5,1)</f>
+        <f>ROUNDDOWN(B5,0)</f>
         <v>0</v>
       </c>
       <c r="CA5">
-        <f>ROUNDUP(B5,0)</f>
+        <f>INT(B5)</f>
         <v>0</v>
       </c>
       <c r="CB5">
-        <f>ROUNDDOWN(B5,0)</f>
+        <f>MOD(A5,3)</f>
         <v>0</v>
       </c>
       <c r="CC5">
-        <f>INT(B5)</f>
+        <f>ABS(A5)</f>
         <v>0</v>
       </c>
       <c r="CD5">
-        <f>MOD(A5,3)</f>
+        <f>SIGN(A5)</f>
         <v>0</v>
       </c>
       <c r="CE5">
-        <f>ABS(A5)</f>
+        <f>SQRT(ABS(A5))</f>
         <v>0</v>
       </c>
       <c r="CF5">
-        <f>SIGN(A5)</f>
+        <f>POWER(ABS(A5),2)</f>
         <v>0</v>
       </c>
       <c r="CG5">
-        <f>SQRT(ABS(A5))</f>
+        <f>CEILING(B5,1)</f>
         <v>0</v>
       </c>
       <c r="CH5">
-        <f>POWER(ABS(A5),2)</f>
+        <f>FLOOR(B5,1)</f>
         <v>0</v>
       </c>
       <c r="CI5">
-        <f>CEILING(B5,1)</f>
+        <f>LN(ABS(A5)+1)</f>
         <v>0</v>
       </c>
       <c r="CJ5">
-        <f>FLOOR(B5,1)</f>
+        <f>LOG(ABS(A5)+1,10)</f>
         <v>0</v>
       </c>
       <c r="CK5">
-        <f>LN(ABS(A5)+1)</f>
+        <f>LOG10(ABS(A5)+1)</f>
         <v>0</v>
       </c>
       <c r="CL5">
-        <f>LOG(ABS(A5)+1,10)</f>
+        <f>EXP(1)</f>
         <v>0</v>
       </c>
       <c r="CM5">
-        <f>LOG10(ABS(A5)+1)</f>
+        <f>SIN(B5)</f>
         <v>0</v>
       </c>
       <c r="CN5">
-        <f>EXP(1)</f>
+        <f>COS(B5)</f>
         <v>0</v>
       </c>
       <c r="CO5">
-        <f>SIN(B5)</f>
+        <f>TAN(B5)</f>
         <v>0</v>
       </c>
       <c r="CP5">
-        <f>COS(B5)</f>
+        <f>ASIN(B5/100)</f>
         <v>0</v>
       </c>
       <c r="CQ5">
-        <f>TAN(B5)</f>
+        <f>ACOS(B5/100)</f>
         <v>0</v>
       </c>
       <c r="CR5">
-        <f>ASIN(B5/100)</f>
+        <f>ATAN(B5)</f>
         <v>0</v>
       </c>
       <c r="CS5">
-        <f>ACOS(B5/100)</f>
+        <f>ATAN2(A5,B5)</f>
         <v>0</v>
       </c>
       <c r="CT5">
-        <f>ATAN(B5)</f>
+        <f>PI()</f>
         <v>0</v>
       </c>
       <c r="CU5">
-        <f>ATAN2(A5,B5)</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
       <c r="CV5">
-        <f>PI()</f>
+        <f>NOW()</f>
         <v>0</v>
       </c>
       <c r="CW5">
-        <f>TODAY()</f>
+        <f>DATE(2026,4,20)</f>
         <v>0</v>
       </c>
       <c r="CX5">
-        <f>NOW()</f>
+        <f>YEAR(G5)</f>
         <v>0</v>
       </c>
       <c r="CY5">
-        <f>DATE(2026,4,20)</f>
+        <f>MONTH(G5)</f>
         <v>0</v>
       </c>
       <c r="CZ5">
-        <f>YEAR(G5)</f>
+        <f>DAY(G5)</f>
         <v>0</v>
       </c>
       <c r="DA5">
-        <f>MONTH(G5)</f>
+        <f>WEEKDAY(G5)</f>
         <v>0</v>
       </c>
       <c r="DB5">
-        <f>DAY(G5)</f>
+        <f>EDATE(G5,3)</f>
         <v>0</v>
       </c>
       <c r="DC5">
-        <f>WEEKDAY(G5)</f>
+        <f>EOMONTH(G5,0)</f>
         <v>0</v>
       </c>
       <c r="DD5">
-        <f>EDATE(G5,3)</f>
+        <f>DATEDIF(DATE(2020,1,1),G5,"d")</f>
         <v>0</v>
       </c>
       <c r="DE5">
-        <f>EOMONTH(G5,0)</f>
+        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
         <v>0</v>
       </c>
       <c r="DF5">
-        <f>DATEDIF(DATE(2020,1,1),G5,"d")</f>
+        <f>WORKDAY(DATE(2026,1,1),10)</f>
         <v>0</v>
       </c>
       <c r="DG5">
-        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
+        <f>ISBLANK(H5)</f>
         <v>0</v>
       </c>
       <c r="DH5">
-        <f>WORKDAY(DATE(2026,1,1),10)</f>
+        <f>ISNUMBER(A5)</f>
         <v>0</v>
       </c>
       <c r="DI5">
-        <f>ISBLANK(H5)</f>
+        <f>ISTEXT(F5)</f>
         <v>0</v>
       </c>
       <c r="DJ5">
-        <f>ISNUMBER(A5)</f>
+        <f>ISLOGICAL(D5)</f>
         <v>0</v>
       </c>
       <c r="DK5">
-        <f>ISTEXT(F5)</f>
+        <f>ISNONTEXT(A5)</f>
         <v>0</v>
       </c>
       <c r="DL5">
-        <f>ISLOGICAL(D5)</f>
+        <f>ISERROR(1/0)</f>
         <v>0</v>
       </c>
       <c r="DM5">
-        <f>ISNONTEXT(A5)</f>
+        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="DN5">
-        <f>ISERROR(1/0)</f>
+        <f>ISREF(A5)</f>
         <v>0</v>
       </c>
       <c r="DO5">
-        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
+        <f>NA()</f>
         <v>0</v>
       </c>
       <c r="DP5">
-        <f>ISREF(A5)</f>
+        <f>TYPE(A5)</f>
         <v>0</v>
       </c>
       <c r="DQ5">
-        <f>NA()</f>
+        <f>PMT(0.05/12,360,-200000)</f>
         <v>0</v>
       </c>
       <c r="DR5">
-        <f>TYPE(A5)</f>
+        <f>PV(0.08/12,120,-500)</f>
         <v>0</v>
       </c>
       <c r="DS5">
-        <f>PMT(0.05/12,360,-200000)</f>
+        <f>FV(0.06/12,240,-200)</f>
         <v>0</v>
       </c>
       <c r="DT5">
-        <f>PV(0.08/12,120,-500)</f>
+        <f>NPV(0.1,A5,B5,C5)</f>
         <v>0</v>
       </c>
       <c r="DU5">
-        <f>FV(0.06/12,240,-200)</f>
-        <v>0</v>
-      </c>
-      <c r="DV5">
-        <f>NPV(0.1,A5,B5,C5)</f>
-        <v>0</v>
-      </c>
-      <c r="DW5">
         <f>RATE(120,-500,50000)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:127">
+    <row r="6" spans="1:125">
       <c r="A6">
         <v>-5.0</v>
       </c>
@@ -3504,7 +3460,7 @@
         <v>2</v>
       </c>
       <c r="F6" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G6" s="1">
         <v>45200.0</v>
@@ -3677,319 +3633,311 @@
         <v>0</v>
       </c>
       <c r="AX6">
-        <f>_xlfn.MINIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
+        <f>VLOOKUP(E6,Lookup1!A:C,2,FALSE)</f>
         <v>0</v>
       </c>
       <c r="AY6">
-        <f>_xlfn.MAXIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
-        <v>0</v>
-      </c>
-      <c r="AZ6">
-        <f>VLOOKUP(E6,Lookup1!A:C,2,FALSE)</f>
+        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ6" cm="1">
+        <f t="array" ref="AZ6">_xlfn.XLOOKUP(E6,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
         <v>0</v>
       </c>
       <c r="BA6">
-        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BB6" cm="1">
-        <f t="array" ref="BB6">_xlfn.XLOOKUP(E6,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
+        <f>MATCH(E6,Lookup1!A:A,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BB6">
+        <f>_xlfn.XMATCH(E6,Lookup1!A:A,0)</f>
         <v>0</v>
       </c>
       <c r="BC6">
-        <f>MATCH(E6,Lookup1!A:A,0)</f>
+        <f>INDEX(Lookup1!B:B,MATCH(E6,Lookup1!A:A,0))</f>
         <v>0</v>
       </c>
       <c r="BD6">
-        <f>_xlfn.XMATCH(E6,Lookup1!A:A,0)</f>
+        <f>CHOOSE(2,"alpha","beta","gamma")</f>
         <v>0</v>
       </c>
       <c r="BE6">
-        <f>INDEX(Lookup1!B:B,MATCH(E6,Lookup1!A:A,0))</f>
+        <f>LEFT(F6,3)</f>
         <v>0</v>
       </c>
       <c r="BF6">
-        <f>CHOOSE(2,"alpha","beta","gamma")</f>
+        <f>RIGHT(F6,3)</f>
         <v>0</v>
       </c>
       <c r="BG6">
-        <f>LEFT(F6,3)</f>
+        <f>MID(F6,2,3)</f>
         <v>0</v>
       </c>
       <c r="BH6">
-        <f>RIGHT(F6,3)</f>
+        <f>LEN(F6)</f>
         <v>0</v>
       </c>
       <c r="BI6">
-        <f>MID(F6,2,3)</f>
+        <f>UPPER(F6)</f>
         <v>0</v>
       </c>
       <c r="BJ6">
-        <f>LEN(F6)</f>
+        <f>LOWER(F6)</f>
         <v>0</v>
       </c>
       <c r="BK6">
-        <f>UPPER(F6)</f>
+        <f>PROPER(F6)</f>
         <v>0</v>
       </c>
       <c r="BL6">
-        <f>LOWER(F6)</f>
+        <f>TRIM(F6)</f>
         <v>0</v>
       </c>
       <c r="BM6">
-        <f>PROPER(F6)</f>
+        <f>CLEAN(F6)</f>
         <v>0</v>
       </c>
       <c r="BN6">
-        <f>TRIM(F6)</f>
+        <f>_xlfn.CONCAT(E6,"-",F6)</f>
         <v>0</v>
       </c>
       <c r="BO6">
-        <f>CLEAN(F6)</f>
+        <f>CONCATENATE(E6,"-",F6)</f>
         <v>0</v>
       </c>
       <c r="BP6">
-        <f>_xlfn.CONCAT(E6,"-",F6)</f>
+        <f>_xlfn.TEXTJOIN("-",TRUE,E6,F6)</f>
         <v>0</v>
       </c>
       <c r="BQ6">
-        <f>CONCATENATE(E6,"-",F6)</f>
+        <f>IFERROR(FIND("l",F6),0)</f>
         <v>0</v>
       </c>
       <c r="BR6">
-        <f>_xlfn.TEXTJOIN("-",TRUE,E6,F6)</f>
+        <f>IFERROR(SEARCH("L",F6),0)</f>
         <v>0</v>
       </c>
       <c r="BS6">
-        <f>IFERROR(FIND("l",F6),0)</f>
+        <f>SUBSTITUTE(F6,"o","0")</f>
         <v>0</v>
       </c>
       <c r="BT6">
-        <f>IFERROR(SEARCH("L",F6),0)</f>
+        <f>REPLACE(F6,1,1,"X")</f>
         <v>0</v>
       </c>
       <c r="BU6">
-        <f>SUBSTITUTE(F6,"o","0")</f>
+        <f>TEXT(C6,"0.00")</f>
         <v>0</v>
       </c>
       <c r="BV6">
-        <f>REPLACE(F6,1,1,"X")</f>
+        <f>VALUE("123.45")</f>
         <v>0</v>
       </c>
       <c r="BW6">
-        <f>TEXT(C6,"0.00")</f>
+        <f>EXACT(F6,"hello")</f>
         <v>0</v>
       </c>
       <c r="BX6">
-        <f>VALUE("123.45")</f>
+        <f>ROUND(B6,1)</f>
         <v>0</v>
       </c>
       <c r="BY6">
-        <f>EXACT(F6,"hello")</f>
+        <f>ROUNDUP(B6,0)</f>
         <v>0</v>
       </c>
       <c r="BZ6">
-        <f>ROUND(B6,1)</f>
+        <f>ROUNDDOWN(B6,0)</f>
         <v>0</v>
       </c>
       <c r="CA6">
-        <f>ROUNDUP(B6,0)</f>
+        <f>INT(B6)</f>
         <v>0</v>
       </c>
       <c r="CB6">
-        <f>ROUNDDOWN(B6,0)</f>
+        <f>MOD(A6,3)</f>
         <v>0</v>
       </c>
       <c r="CC6">
-        <f>INT(B6)</f>
+        <f>ABS(A6)</f>
         <v>0</v>
       </c>
       <c r="CD6">
-        <f>MOD(A6,3)</f>
+        <f>SIGN(A6)</f>
         <v>0</v>
       </c>
       <c r="CE6">
-        <f>ABS(A6)</f>
+        <f>SQRT(ABS(A6))</f>
         <v>0</v>
       </c>
       <c r="CF6">
-        <f>SIGN(A6)</f>
+        <f>POWER(ABS(A6),2)</f>
         <v>0</v>
       </c>
       <c r="CG6">
-        <f>SQRT(ABS(A6))</f>
+        <f>CEILING(B6,1)</f>
         <v>0</v>
       </c>
       <c r="CH6">
-        <f>POWER(ABS(A6),2)</f>
+        <f>FLOOR(B6,1)</f>
         <v>0</v>
       </c>
       <c r="CI6">
-        <f>CEILING(B6,1)</f>
+        <f>LN(ABS(A6)+1)</f>
         <v>0</v>
       </c>
       <c r="CJ6">
-        <f>FLOOR(B6,1)</f>
+        <f>LOG(ABS(A6)+1,10)</f>
         <v>0</v>
       </c>
       <c r="CK6">
-        <f>LN(ABS(A6)+1)</f>
+        <f>LOG10(ABS(A6)+1)</f>
         <v>0</v>
       </c>
       <c r="CL6">
-        <f>LOG(ABS(A6)+1,10)</f>
+        <f>EXP(1)</f>
         <v>0</v>
       </c>
       <c r="CM6">
-        <f>LOG10(ABS(A6)+1)</f>
+        <f>SIN(B6)</f>
         <v>0</v>
       </c>
       <c r="CN6">
-        <f>EXP(1)</f>
+        <f>COS(B6)</f>
         <v>0</v>
       </c>
       <c r="CO6">
-        <f>SIN(B6)</f>
+        <f>TAN(B6)</f>
         <v>0</v>
       </c>
       <c r="CP6">
-        <f>COS(B6)</f>
+        <f>ASIN(B6/100)</f>
         <v>0</v>
       </c>
       <c r="CQ6">
-        <f>TAN(B6)</f>
+        <f>ACOS(B6/100)</f>
         <v>0</v>
       </c>
       <c r="CR6">
-        <f>ASIN(B6/100)</f>
+        <f>ATAN(B6)</f>
         <v>0</v>
       </c>
       <c r="CS6">
-        <f>ACOS(B6/100)</f>
+        <f>ATAN2(A6,B6)</f>
         <v>0</v>
       </c>
       <c r="CT6">
-        <f>ATAN(B6)</f>
+        <f>PI()</f>
         <v>0</v>
       </c>
       <c r="CU6">
-        <f>ATAN2(A6,B6)</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
       <c r="CV6">
-        <f>PI()</f>
+        <f>NOW()</f>
         <v>0</v>
       </c>
       <c r="CW6">
-        <f>TODAY()</f>
+        <f>DATE(2026,4,20)</f>
         <v>0</v>
       </c>
       <c r="CX6">
-        <f>NOW()</f>
+        <f>YEAR(G6)</f>
         <v>0</v>
       </c>
       <c r="CY6">
-        <f>DATE(2026,4,20)</f>
+        <f>MONTH(G6)</f>
         <v>0</v>
       </c>
       <c r="CZ6">
-        <f>YEAR(G6)</f>
+        <f>DAY(G6)</f>
         <v>0</v>
       </c>
       <c r="DA6">
-        <f>MONTH(G6)</f>
+        <f>WEEKDAY(G6)</f>
         <v>0</v>
       </c>
       <c r="DB6">
-        <f>DAY(G6)</f>
+        <f>EDATE(G6,3)</f>
         <v>0</v>
       </c>
       <c r="DC6">
-        <f>WEEKDAY(G6)</f>
+        <f>EOMONTH(G6,0)</f>
         <v>0</v>
       </c>
       <c r="DD6">
-        <f>EDATE(G6,3)</f>
+        <f>DATEDIF(DATE(2020,1,1),G6,"d")</f>
         <v>0</v>
       </c>
       <c r="DE6">
-        <f>EOMONTH(G6,0)</f>
+        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
         <v>0</v>
       </c>
       <c r="DF6">
-        <f>DATEDIF(DATE(2020,1,1),G6,"d")</f>
+        <f>WORKDAY(DATE(2026,1,1),10)</f>
         <v>0</v>
       </c>
       <c r="DG6">
-        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
+        <f>ISBLANK(H6)</f>
         <v>0</v>
       </c>
       <c r="DH6">
-        <f>WORKDAY(DATE(2026,1,1),10)</f>
+        <f>ISNUMBER(A6)</f>
         <v>0</v>
       </c>
       <c r="DI6">
-        <f>ISBLANK(H6)</f>
+        <f>ISTEXT(F6)</f>
         <v>0</v>
       </c>
       <c r="DJ6">
-        <f>ISNUMBER(A6)</f>
+        <f>ISLOGICAL(D6)</f>
         <v>0</v>
       </c>
       <c r="DK6">
-        <f>ISTEXT(F6)</f>
+        <f>ISNONTEXT(A6)</f>
         <v>0</v>
       </c>
       <c r="DL6">
-        <f>ISLOGICAL(D6)</f>
+        <f>ISERROR(1/0)</f>
         <v>0</v>
       </c>
       <c r="DM6">
-        <f>ISNONTEXT(A6)</f>
+        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="DN6">
-        <f>ISERROR(1/0)</f>
+        <f>ISREF(A6)</f>
         <v>0</v>
       </c>
       <c r="DO6">
-        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
+        <f>NA()</f>
         <v>0</v>
       </c>
       <c r="DP6">
-        <f>ISREF(A6)</f>
+        <f>TYPE(A6)</f>
         <v>0</v>
       </c>
       <c r="DQ6">
-        <f>NA()</f>
+        <f>PMT(0.05/12,360,-200000)</f>
         <v>0</v>
       </c>
       <c r="DR6">
-        <f>TYPE(A6)</f>
+        <f>PV(0.08/12,120,-500)</f>
         <v>0</v>
       </c>
       <c r="DS6">
-        <f>PMT(0.05/12,360,-200000)</f>
+        <f>FV(0.06/12,240,-200)</f>
         <v>0</v>
       </c>
       <c r="DT6">
-        <f>PV(0.08/12,120,-500)</f>
+        <f>NPV(0.1,A6,B6,C6)</f>
         <v>0</v>
       </c>
       <c r="DU6">
-        <f>FV(0.06/12,240,-200)</f>
-        <v>0</v>
-      </c>
-      <c r="DV6">
-        <f>NPV(0.1,A6,B6,C6)</f>
-        <v>0</v>
-      </c>
-      <c r="DW6">
         <f>RATE(120,-500,50000)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:127">
+    <row r="7" spans="1:125">
       <c r="A7">
         <v>50.0</v>
       </c>
@@ -4006,7 +3954,7 @@
         <v>4</v>
       </c>
       <c r="F7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="G7" s="1">
         <v>45300.0</v>
@@ -4179,319 +4127,311 @@
         <v>0</v>
       </c>
       <c r="AX7">
-        <f>_xlfn.MINIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
+        <f>VLOOKUP(E7,Lookup1!A:C,2,FALSE)</f>
         <v>0</v>
       </c>
       <c r="AY7">
-        <f>_xlfn.MAXIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
-        <v>0</v>
-      </c>
-      <c r="AZ7">
-        <f>VLOOKUP(E7,Lookup1!A:C,2,FALSE)</f>
+        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ7" cm="1">
+        <f t="array" ref="AZ7">_xlfn.XLOOKUP(E7,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
         <v>0</v>
       </c>
       <c r="BA7">
-        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BB7" cm="1">
-        <f t="array" ref="BB7">_xlfn.XLOOKUP(E7,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
+        <f>MATCH(E7,Lookup1!A:A,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BB7">
+        <f>_xlfn.XMATCH(E7,Lookup1!A:A,0)</f>
         <v>0</v>
       </c>
       <c r="BC7">
-        <f>MATCH(E7,Lookup1!A:A,0)</f>
+        <f>INDEX(Lookup1!B:B,MATCH(E7,Lookup1!A:A,0))</f>
         <v>0</v>
       </c>
       <c r="BD7">
-        <f>_xlfn.XMATCH(E7,Lookup1!A:A,0)</f>
+        <f>CHOOSE(2,"alpha","beta","gamma")</f>
         <v>0</v>
       </c>
       <c r="BE7">
-        <f>INDEX(Lookup1!B:B,MATCH(E7,Lookup1!A:A,0))</f>
+        <f>LEFT(F7,3)</f>
         <v>0</v>
       </c>
       <c r="BF7">
-        <f>CHOOSE(2,"alpha","beta","gamma")</f>
+        <f>RIGHT(F7,3)</f>
         <v>0</v>
       </c>
       <c r="BG7">
-        <f>LEFT(F7,3)</f>
+        <f>MID(F7,2,3)</f>
         <v>0</v>
       </c>
       <c r="BH7">
-        <f>RIGHT(F7,3)</f>
+        <f>LEN(F7)</f>
         <v>0</v>
       </c>
       <c r="BI7">
-        <f>MID(F7,2,3)</f>
+        <f>UPPER(F7)</f>
         <v>0</v>
       </c>
       <c r="BJ7">
-        <f>LEN(F7)</f>
+        <f>LOWER(F7)</f>
         <v>0</v>
       </c>
       <c r="BK7">
-        <f>UPPER(F7)</f>
+        <f>PROPER(F7)</f>
         <v>0</v>
       </c>
       <c r="BL7">
-        <f>LOWER(F7)</f>
+        <f>TRIM(F7)</f>
         <v>0</v>
       </c>
       <c r="BM7">
-        <f>PROPER(F7)</f>
+        <f>CLEAN(F7)</f>
         <v>0</v>
       </c>
       <c r="BN7">
-        <f>TRIM(F7)</f>
+        <f>_xlfn.CONCAT(E7,"-",F7)</f>
         <v>0</v>
       </c>
       <c r="BO7">
-        <f>CLEAN(F7)</f>
+        <f>CONCATENATE(E7,"-",F7)</f>
         <v>0</v>
       </c>
       <c r="BP7">
-        <f>_xlfn.CONCAT(E7,"-",F7)</f>
+        <f>_xlfn.TEXTJOIN("-",TRUE,E7,F7)</f>
         <v>0</v>
       </c>
       <c r="BQ7">
-        <f>CONCATENATE(E7,"-",F7)</f>
+        <f>IFERROR(FIND("l",F7),0)</f>
         <v>0</v>
       </c>
       <c r="BR7">
-        <f>_xlfn.TEXTJOIN("-",TRUE,E7,F7)</f>
+        <f>IFERROR(SEARCH("L",F7),0)</f>
         <v>0</v>
       </c>
       <c r="BS7">
-        <f>IFERROR(FIND("l",F7),0)</f>
+        <f>SUBSTITUTE(F7,"o","0")</f>
         <v>0</v>
       </c>
       <c r="BT7">
-        <f>IFERROR(SEARCH("L",F7),0)</f>
+        <f>REPLACE(F7,1,1,"X")</f>
         <v>0</v>
       </c>
       <c r="BU7">
-        <f>SUBSTITUTE(F7,"o","0")</f>
+        <f>TEXT(C7,"0.00")</f>
         <v>0</v>
       </c>
       <c r="BV7">
-        <f>REPLACE(F7,1,1,"X")</f>
+        <f>VALUE("123.45")</f>
         <v>0</v>
       </c>
       <c r="BW7">
-        <f>TEXT(C7,"0.00")</f>
+        <f>EXACT(F7,"hello")</f>
         <v>0</v>
       </c>
       <c r="BX7">
-        <f>VALUE("123.45")</f>
+        <f>ROUND(B7,1)</f>
         <v>0</v>
       </c>
       <c r="BY7">
-        <f>EXACT(F7,"hello")</f>
+        <f>ROUNDUP(B7,0)</f>
         <v>0</v>
       </c>
       <c r="BZ7">
-        <f>ROUND(B7,1)</f>
+        <f>ROUNDDOWN(B7,0)</f>
         <v>0</v>
       </c>
       <c r="CA7">
-        <f>ROUNDUP(B7,0)</f>
+        <f>INT(B7)</f>
         <v>0</v>
       </c>
       <c r="CB7">
-        <f>ROUNDDOWN(B7,0)</f>
+        <f>MOD(A7,3)</f>
         <v>0</v>
       </c>
       <c r="CC7">
-        <f>INT(B7)</f>
+        <f>ABS(A7)</f>
         <v>0</v>
       </c>
       <c r="CD7">
-        <f>MOD(A7,3)</f>
+        <f>SIGN(A7)</f>
         <v>0</v>
       </c>
       <c r="CE7">
-        <f>ABS(A7)</f>
+        <f>SQRT(ABS(A7))</f>
         <v>0</v>
       </c>
       <c r="CF7">
-        <f>SIGN(A7)</f>
+        <f>POWER(ABS(A7),2)</f>
         <v>0</v>
       </c>
       <c r="CG7">
-        <f>SQRT(ABS(A7))</f>
+        <f>CEILING(B7,1)</f>
         <v>0</v>
       </c>
       <c r="CH7">
-        <f>POWER(ABS(A7),2)</f>
+        <f>FLOOR(B7,1)</f>
         <v>0</v>
       </c>
       <c r="CI7">
-        <f>CEILING(B7,1)</f>
+        <f>LN(ABS(A7)+1)</f>
         <v>0</v>
       </c>
       <c r="CJ7">
-        <f>FLOOR(B7,1)</f>
+        <f>LOG(ABS(A7)+1,10)</f>
         <v>0</v>
       </c>
       <c r="CK7">
-        <f>LN(ABS(A7)+1)</f>
+        <f>LOG10(ABS(A7)+1)</f>
         <v>0</v>
       </c>
       <c r="CL7">
-        <f>LOG(ABS(A7)+1,10)</f>
+        <f>EXP(1)</f>
         <v>0</v>
       </c>
       <c r="CM7">
-        <f>LOG10(ABS(A7)+1)</f>
+        <f>SIN(B7)</f>
         <v>0</v>
       </c>
       <c r="CN7">
-        <f>EXP(1)</f>
+        <f>COS(B7)</f>
         <v>0</v>
       </c>
       <c r="CO7">
-        <f>SIN(B7)</f>
+        <f>TAN(B7)</f>
         <v>0</v>
       </c>
       <c r="CP7">
-        <f>COS(B7)</f>
+        <f>ASIN(B7/100)</f>
         <v>0</v>
       </c>
       <c r="CQ7">
-        <f>TAN(B7)</f>
+        <f>ACOS(B7/100)</f>
         <v>0</v>
       </c>
       <c r="CR7">
-        <f>ASIN(B7/100)</f>
+        <f>ATAN(B7)</f>
         <v>0</v>
       </c>
       <c r="CS7">
-        <f>ACOS(B7/100)</f>
+        <f>ATAN2(A7,B7)</f>
         <v>0</v>
       </c>
       <c r="CT7">
-        <f>ATAN(B7)</f>
+        <f>PI()</f>
         <v>0</v>
       </c>
       <c r="CU7">
-        <f>ATAN2(A7,B7)</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
       <c r="CV7">
-        <f>PI()</f>
+        <f>NOW()</f>
         <v>0</v>
       </c>
       <c r="CW7">
-        <f>TODAY()</f>
+        <f>DATE(2026,4,20)</f>
         <v>0</v>
       </c>
       <c r="CX7">
-        <f>NOW()</f>
+        <f>YEAR(G7)</f>
         <v>0</v>
       </c>
       <c r="CY7">
-        <f>DATE(2026,4,20)</f>
+        <f>MONTH(G7)</f>
         <v>0</v>
       </c>
       <c r="CZ7">
-        <f>YEAR(G7)</f>
+        <f>DAY(G7)</f>
         <v>0</v>
       </c>
       <c r="DA7">
-        <f>MONTH(G7)</f>
+        <f>WEEKDAY(G7)</f>
         <v>0</v>
       </c>
       <c r="DB7">
-        <f>DAY(G7)</f>
+        <f>EDATE(G7,3)</f>
         <v>0</v>
       </c>
       <c r="DC7">
-        <f>WEEKDAY(G7)</f>
+        <f>EOMONTH(G7,0)</f>
         <v>0</v>
       </c>
       <c r="DD7">
-        <f>EDATE(G7,3)</f>
+        <f>DATEDIF(DATE(2020,1,1),G7,"d")</f>
         <v>0</v>
       </c>
       <c r="DE7">
-        <f>EOMONTH(G7,0)</f>
+        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
         <v>0</v>
       </c>
       <c r="DF7">
-        <f>DATEDIF(DATE(2020,1,1),G7,"d")</f>
+        <f>WORKDAY(DATE(2026,1,1),10)</f>
         <v>0</v>
       </c>
       <c r="DG7">
-        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
+        <f>ISBLANK(H7)</f>
         <v>0</v>
       </c>
       <c r="DH7">
-        <f>WORKDAY(DATE(2026,1,1),10)</f>
+        <f>ISNUMBER(A7)</f>
         <v>0</v>
       </c>
       <c r="DI7">
-        <f>ISBLANK(H7)</f>
+        <f>ISTEXT(F7)</f>
         <v>0</v>
       </c>
       <c r="DJ7">
-        <f>ISNUMBER(A7)</f>
+        <f>ISLOGICAL(D7)</f>
         <v>0</v>
       </c>
       <c r="DK7">
-        <f>ISTEXT(F7)</f>
+        <f>ISNONTEXT(A7)</f>
         <v>0</v>
       </c>
       <c r="DL7">
-        <f>ISLOGICAL(D7)</f>
+        <f>ISERROR(1/0)</f>
         <v>0</v>
       </c>
       <c r="DM7">
-        <f>ISNONTEXT(A7)</f>
+        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="DN7">
-        <f>ISERROR(1/0)</f>
+        <f>ISREF(A7)</f>
         <v>0</v>
       </c>
       <c r="DO7">
-        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
+        <f>NA()</f>
         <v>0</v>
       </c>
       <c r="DP7">
-        <f>ISREF(A7)</f>
+        <f>TYPE(A7)</f>
         <v>0</v>
       </c>
       <c r="DQ7">
-        <f>NA()</f>
+        <f>PMT(0.05/12,360,-200000)</f>
         <v>0</v>
       </c>
       <c r="DR7">
-        <f>TYPE(A7)</f>
+        <f>PV(0.08/12,120,-500)</f>
         <v>0</v>
       </c>
       <c r="DS7">
-        <f>PMT(0.05/12,360,-200000)</f>
+        <f>FV(0.06/12,240,-200)</f>
         <v>0</v>
       </c>
       <c r="DT7">
-        <f>PV(0.08/12,120,-500)</f>
+        <f>NPV(0.1,A7,B7,C7)</f>
         <v>0</v>
       </c>
       <c r="DU7">
-        <f>FV(0.06/12,240,-200)</f>
-        <v>0</v>
-      </c>
-      <c r="DV7">
-        <f>NPV(0.1,A7,B7,C7)</f>
-        <v>0</v>
-      </c>
-      <c r="DW7">
         <f>RATE(120,-500,50000)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:127">
+    <row r="8" spans="1:125">
       <c r="A8">
         <v>75.0</v>
       </c>
@@ -4508,7 +4448,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G8" s="1">
         <v>44800.0</v>
@@ -4678,319 +4618,311 @@
         <v>0</v>
       </c>
       <c r="AX8">
-        <f>_xlfn.MINIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
+        <f>VLOOKUP(E8,Lookup1!A:C,2,FALSE)</f>
         <v>0</v>
       </c>
       <c r="AY8">
-        <f>_xlfn.MAXIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
-        <v>0</v>
-      </c>
-      <c r="AZ8">
-        <f>VLOOKUP(E8,Lookup1!A:C,2,FALSE)</f>
+        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ8" cm="1">
+        <f t="array" ref="AZ8">_xlfn.XLOOKUP(E8,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
         <v>0</v>
       </c>
       <c r="BA8">
-        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BB8" cm="1">
-        <f t="array" ref="BB8">_xlfn.XLOOKUP(E8,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
+        <f>MATCH(E8,Lookup1!A:A,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BB8">
+        <f>_xlfn.XMATCH(E8,Lookup1!A:A,0)</f>
         <v>0</v>
       </c>
       <c r="BC8">
-        <f>MATCH(E8,Lookup1!A:A,0)</f>
+        <f>INDEX(Lookup1!B:B,MATCH(E8,Lookup1!A:A,0))</f>
         <v>0</v>
       </c>
       <c r="BD8">
-        <f>_xlfn.XMATCH(E8,Lookup1!A:A,0)</f>
+        <f>CHOOSE(2,"alpha","beta","gamma")</f>
         <v>0</v>
       </c>
       <c r="BE8">
-        <f>INDEX(Lookup1!B:B,MATCH(E8,Lookup1!A:A,0))</f>
+        <f>LEFT(F8,3)</f>
         <v>0</v>
       </c>
       <c r="BF8">
-        <f>CHOOSE(2,"alpha","beta","gamma")</f>
+        <f>RIGHT(F8,3)</f>
         <v>0</v>
       </c>
       <c r="BG8">
-        <f>LEFT(F8,3)</f>
+        <f>MID(F8,2,3)</f>
         <v>0</v>
       </c>
       <c r="BH8">
-        <f>RIGHT(F8,3)</f>
+        <f>LEN(F8)</f>
         <v>0</v>
       </c>
       <c r="BI8">
-        <f>MID(F8,2,3)</f>
+        <f>UPPER(F8)</f>
         <v>0</v>
       </c>
       <c r="BJ8">
-        <f>LEN(F8)</f>
+        <f>LOWER(F8)</f>
         <v>0</v>
       </c>
       <c r="BK8">
-        <f>UPPER(F8)</f>
+        <f>PROPER(F8)</f>
         <v>0</v>
       </c>
       <c r="BL8">
-        <f>LOWER(F8)</f>
+        <f>TRIM(F8)</f>
         <v>0</v>
       </c>
       <c r="BM8">
-        <f>PROPER(F8)</f>
+        <f>CLEAN(F8)</f>
         <v>0</v>
       </c>
       <c r="BN8">
-        <f>TRIM(F8)</f>
+        <f>_xlfn.CONCAT(E8,"-",F8)</f>
         <v>0</v>
       </c>
       <c r="BO8">
-        <f>CLEAN(F8)</f>
+        <f>CONCATENATE(E8,"-",F8)</f>
         <v>0</v>
       </c>
       <c r="BP8">
-        <f>_xlfn.CONCAT(E8,"-",F8)</f>
+        <f>_xlfn.TEXTJOIN("-",TRUE,E8,F8)</f>
         <v>0</v>
       </c>
       <c r="BQ8">
-        <f>CONCATENATE(E8,"-",F8)</f>
+        <f>IFERROR(FIND("l",F8),0)</f>
         <v>0</v>
       </c>
       <c r="BR8">
-        <f>_xlfn.TEXTJOIN("-",TRUE,E8,F8)</f>
+        <f>IFERROR(SEARCH("L",F8),0)</f>
         <v>0</v>
       </c>
       <c r="BS8">
-        <f>IFERROR(FIND("l",F8),0)</f>
+        <f>SUBSTITUTE(F8,"o","0")</f>
         <v>0</v>
       </c>
       <c r="BT8">
-        <f>IFERROR(SEARCH("L",F8),0)</f>
+        <f>REPLACE(F8,1,1,"X")</f>
         <v>0</v>
       </c>
       <c r="BU8">
-        <f>SUBSTITUTE(F8,"o","0")</f>
+        <f>TEXT(C8,"0.00")</f>
         <v>0</v>
       </c>
       <c r="BV8">
-        <f>REPLACE(F8,1,1,"X")</f>
+        <f>VALUE("123.45")</f>
         <v>0</v>
       </c>
       <c r="BW8">
-        <f>TEXT(C8,"0.00")</f>
+        <f>EXACT(F8,"hello")</f>
         <v>0</v>
       </c>
       <c r="BX8">
-        <f>VALUE("123.45")</f>
+        <f>ROUND(B8,1)</f>
         <v>0</v>
       </c>
       <c r="BY8">
-        <f>EXACT(F8,"hello")</f>
+        <f>ROUNDUP(B8,0)</f>
         <v>0</v>
       </c>
       <c r="BZ8">
-        <f>ROUND(B8,1)</f>
+        <f>ROUNDDOWN(B8,0)</f>
         <v>0</v>
       </c>
       <c r="CA8">
-        <f>ROUNDUP(B8,0)</f>
+        <f>INT(B8)</f>
         <v>0</v>
       </c>
       <c r="CB8">
-        <f>ROUNDDOWN(B8,0)</f>
+        <f>MOD(A8,3)</f>
         <v>0</v>
       </c>
       <c r="CC8">
-        <f>INT(B8)</f>
+        <f>ABS(A8)</f>
         <v>0</v>
       </c>
       <c r="CD8">
-        <f>MOD(A8,3)</f>
+        <f>SIGN(A8)</f>
         <v>0</v>
       </c>
       <c r="CE8">
-        <f>ABS(A8)</f>
+        <f>SQRT(ABS(A8))</f>
         <v>0</v>
       </c>
       <c r="CF8">
-        <f>SIGN(A8)</f>
+        <f>POWER(ABS(A8),2)</f>
         <v>0</v>
       </c>
       <c r="CG8">
-        <f>SQRT(ABS(A8))</f>
+        <f>CEILING(B8,1)</f>
         <v>0</v>
       </c>
       <c r="CH8">
-        <f>POWER(ABS(A8),2)</f>
+        <f>FLOOR(B8,1)</f>
         <v>0</v>
       </c>
       <c r="CI8">
-        <f>CEILING(B8,1)</f>
+        <f>LN(ABS(A8)+1)</f>
         <v>0</v>
       </c>
       <c r="CJ8">
-        <f>FLOOR(B8,1)</f>
+        <f>LOG(ABS(A8)+1,10)</f>
         <v>0</v>
       </c>
       <c r="CK8">
-        <f>LN(ABS(A8)+1)</f>
+        <f>LOG10(ABS(A8)+1)</f>
         <v>0</v>
       </c>
       <c r="CL8">
-        <f>LOG(ABS(A8)+1,10)</f>
+        <f>EXP(1)</f>
         <v>0</v>
       </c>
       <c r="CM8">
-        <f>LOG10(ABS(A8)+1)</f>
+        <f>SIN(B8)</f>
         <v>0</v>
       </c>
       <c r="CN8">
-        <f>EXP(1)</f>
+        <f>COS(B8)</f>
         <v>0</v>
       </c>
       <c r="CO8">
-        <f>SIN(B8)</f>
+        <f>TAN(B8)</f>
         <v>0</v>
       </c>
       <c r="CP8">
-        <f>COS(B8)</f>
+        <f>ASIN(B8/100)</f>
         <v>0</v>
       </c>
       <c r="CQ8">
-        <f>TAN(B8)</f>
+        <f>ACOS(B8/100)</f>
         <v>0</v>
       </c>
       <c r="CR8">
-        <f>ASIN(B8/100)</f>
+        <f>ATAN(B8)</f>
         <v>0</v>
       </c>
       <c r="CS8">
-        <f>ACOS(B8/100)</f>
+        <f>ATAN2(A8,B8)</f>
         <v>0</v>
       </c>
       <c r="CT8">
-        <f>ATAN(B8)</f>
+        <f>PI()</f>
         <v>0</v>
       </c>
       <c r="CU8">
-        <f>ATAN2(A8,B8)</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
       <c r="CV8">
-        <f>PI()</f>
+        <f>NOW()</f>
         <v>0</v>
       </c>
       <c r="CW8">
-        <f>TODAY()</f>
+        <f>DATE(2026,4,20)</f>
         <v>0</v>
       </c>
       <c r="CX8">
-        <f>NOW()</f>
+        <f>YEAR(G8)</f>
         <v>0</v>
       </c>
       <c r="CY8">
-        <f>DATE(2026,4,20)</f>
+        <f>MONTH(G8)</f>
         <v>0</v>
       </c>
       <c r="CZ8">
-        <f>YEAR(G8)</f>
+        <f>DAY(G8)</f>
         <v>0</v>
       </c>
       <c r="DA8">
-        <f>MONTH(G8)</f>
+        <f>WEEKDAY(G8)</f>
         <v>0</v>
       </c>
       <c r="DB8">
-        <f>DAY(G8)</f>
+        <f>EDATE(G8,3)</f>
         <v>0</v>
       </c>
       <c r="DC8">
-        <f>WEEKDAY(G8)</f>
+        <f>EOMONTH(G8,0)</f>
         <v>0</v>
       </c>
       <c r="DD8">
-        <f>EDATE(G8,3)</f>
+        <f>DATEDIF(DATE(2020,1,1),G8,"d")</f>
         <v>0</v>
       </c>
       <c r="DE8">
-        <f>EOMONTH(G8,0)</f>
+        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
         <v>0</v>
       </c>
       <c r="DF8">
-        <f>DATEDIF(DATE(2020,1,1),G8,"d")</f>
+        <f>WORKDAY(DATE(2026,1,1),10)</f>
         <v>0</v>
       </c>
       <c r="DG8">
-        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
+        <f>ISBLANK(H8)</f>
         <v>0</v>
       </c>
       <c r="DH8">
-        <f>WORKDAY(DATE(2026,1,1),10)</f>
+        <f>ISNUMBER(A8)</f>
         <v>0</v>
       </c>
       <c r="DI8">
-        <f>ISBLANK(H8)</f>
+        <f>ISTEXT(F8)</f>
         <v>0</v>
       </c>
       <c r="DJ8">
-        <f>ISNUMBER(A8)</f>
+        <f>ISLOGICAL(D8)</f>
         <v>0</v>
       </c>
       <c r="DK8">
-        <f>ISTEXT(F8)</f>
+        <f>ISNONTEXT(A8)</f>
         <v>0</v>
       </c>
       <c r="DL8">
-        <f>ISLOGICAL(D8)</f>
+        <f>ISERROR(1/0)</f>
         <v>0</v>
       </c>
       <c r="DM8">
-        <f>ISNONTEXT(A8)</f>
+        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="DN8">
-        <f>ISERROR(1/0)</f>
+        <f>ISREF(A8)</f>
         <v>0</v>
       </c>
       <c r="DO8">
-        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
+        <f>NA()</f>
         <v>0</v>
       </c>
       <c r="DP8">
-        <f>ISREF(A8)</f>
+        <f>TYPE(A8)</f>
         <v>0</v>
       </c>
       <c r="DQ8">
-        <f>NA()</f>
+        <f>PMT(0.05/12,360,-200000)</f>
         <v>0</v>
       </c>
       <c r="DR8">
-        <f>TYPE(A8)</f>
+        <f>PV(0.08/12,120,-500)</f>
         <v>0</v>
       </c>
       <c r="DS8">
-        <f>PMT(0.05/12,360,-200000)</f>
+        <f>FV(0.06/12,240,-200)</f>
         <v>0</v>
       </c>
       <c r="DT8">
-        <f>PV(0.08/12,120,-500)</f>
+        <f>NPV(0.1,A8,B8,C8)</f>
         <v>0</v>
       </c>
       <c r="DU8">
-        <f>FV(0.06/12,240,-200)</f>
-        <v>0</v>
-      </c>
-      <c r="DV8">
-        <f>NPV(0.1,A8,B8,C8)</f>
-        <v>0</v>
-      </c>
-      <c r="DW8">
         <f>RATE(120,-500,50000)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:127">
+    <row r="9" spans="1:125">
       <c r="A9">
         <v>1.0</v>
       </c>
@@ -5007,13 +4939,13 @@
         <v>2</v>
       </c>
       <c r="F9" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="G9" s="1">
         <v>45100.0</v>
       </c>
       <c r="H9" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="I9">
         <f>A9+B9</f>
@@ -5180,319 +5112,311 @@
         <v>0</v>
       </c>
       <c r="AX9">
-        <f>_xlfn.MINIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
+        <f>VLOOKUP(E9,Lookup1!A:C,2,FALSE)</f>
         <v>0</v>
       </c>
       <c r="AY9">
-        <f>_xlfn.MAXIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
-        <v>0</v>
-      </c>
-      <c r="AZ9">
-        <f>VLOOKUP(E9,Lookup1!A:C,2,FALSE)</f>
+        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ9" cm="1">
+        <f t="array" ref="AZ9">_xlfn.XLOOKUP(E9,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
         <v>0</v>
       </c>
       <c r="BA9">
-        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BB9" cm="1">
-        <f t="array" ref="BB9">_xlfn.XLOOKUP(E9,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
+        <f>MATCH(E9,Lookup1!A:A,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BB9">
+        <f>_xlfn.XMATCH(E9,Lookup1!A:A,0)</f>
         <v>0</v>
       </c>
       <c r="BC9">
-        <f>MATCH(E9,Lookup1!A:A,0)</f>
+        <f>INDEX(Lookup1!B:B,MATCH(E9,Lookup1!A:A,0))</f>
         <v>0</v>
       </c>
       <c r="BD9">
-        <f>_xlfn.XMATCH(E9,Lookup1!A:A,0)</f>
+        <f>CHOOSE(2,"alpha","beta","gamma")</f>
         <v>0</v>
       </c>
       <c r="BE9">
-        <f>INDEX(Lookup1!B:B,MATCH(E9,Lookup1!A:A,0))</f>
+        <f>LEFT(F9,3)</f>
         <v>0</v>
       </c>
       <c r="BF9">
-        <f>CHOOSE(2,"alpha","beta","gamma")</f>
+        <f>RIGHT(F9,3)</f>
         <v>0</v>
       </c>
       <c r="BG9">
-        <f>LEFT(F9,3)</f>
+        <f>MID(F9,2,3)</f>
         <v>0</v>
       </c>
       <c r="BH9">
-        <f>RIGHT(F9,3)</f>
+        <f>LEN(F9)</f>
         <v>0</v>
       </c>
       <c r="BI9">
-        <f>MID(F9,2,3)</f>
+        <f>UPPER(F9)</f>
         <v>0</v>
       </c>
       <c r="BJ9">
-        <f>LEN(F9)</f>
+        <f>LOWER(F9)</f>
         <v>0</v>
       </c>
       <c r="BK9">
-        <f>UPPER(F9)</f>
+        <f>PROPER(F9)</f>
         <v>0</v>
       </c>
       <c r="BL9">
-        <f>LOWER(F9)</f>
+        <f>TRIM(F9)</f>
         <v>0</v>
       </c>
       <c r="BM9">
-        <f>PROPER(F9)</f>
+        <f>CLEAN(F9)</f>
         <v>0</v>
       </c>
       <c r="BN9">
-        <f>TRIM(F9)</f>
+        <f>_xlfn.CONCAT(E9,"-",F9)</f>
         <v>0</v>
       </c>
       <c r="BO9">
-        <f>CLEAN(F9)</f>
+        <f>CONCATENATE(E9,"-",F9)</f>
         <v>0</v>
       </c>
       <c r="BP9">
-        <f>_xlfn.CONCAT(E9,"-",F9)</f>
+        <f>_xlfn.TEXTJOIN("-",TRUE,E9,F9)</f>
         <v>0</v>
       </c>
       <c r="BQ9">
-        <f>CONCATENATE(E9,"-",F9)</f>
+        <f>IFERROR(FIND("l",F9),0)</f>
         <v>0</v>
       </c>
       <c r="BR9">
-        <f>_xlfn.TEXTJOIN("-",TRUE,E9,F9)</f>
+        <f>IFERROR(SEARCH("L",F9),0)</f>
         <v>0</v>
       </c>
       <c r="BS9">
-        <f>IFERROR(FIND("l",F9),0)</f>
+        <f>SUBSTITUTE(F9,"o","0")</f>
         <v>0</v>
       </c>
       <c r="BT9">
-        <f>IFERROR(SEARCH("L",F9),0)</f>
+        <f>REPLACE(F9,1,1,"X")</f>
         <v>0</v>
       </c>
       <c r="BU9">
-        <f>SUBSTITUTE(F9,"o","0")</f>
+        <f>TEXT(C9,"0.00")</f>
         <v>0</v>
       </c>
       <c r="BV9">
-        <f>REPLACE(F9,1,1,"X")</f>
+        <f>VALUE("123.45")</f>
         <v>0</v>
       </c>
       <c r="BW9">
-        <f>TEXT(C9,"0.00")</f>
+        <f>EXACT(F9,"hello")</f>
         <v>0</v>
       </c>
       <c r="BX9">
-        <f>VALUE("123.45")</f>
+        <f>ROUND(B9,1)</f>
         <v>0</v>
       </c>
       <c r="BY9">
-        <f>EXACT(F9,"hello")</f>
+        <f>ROUNDUP(B9,0)</f>
         <v>0</v>
       </c>
       <c r="BZ9">
-        <f>ROUND(B9,1)</f>
+        <f>ROUNDDOWN(B9,0)</f>
         <v>0</v>
       </c>
       <c r="CA9">
-        <f>ROUNDUP(B9,0)</f>
+        <f>INT(B9)</f>
         <v>0</v>
       </c>
       <c r="CB9">
-        <f>ROUNDDOWN(B9,0)</f>
+        <f>MOD(A9,3)</f>
         <v>0</v>
       </c>
       <c r="CC9">
-        <f>INT(B9)</f>
+        <f>ABS(A9)</f>
         <v>0</v>
       </c>
       <c r="CD9">
-        <f>MOD(A9,3)</f>
+        <f>SIGN(A9)</f>
         <v>0</v>
       </c>
       <c r="CE9">
-        <f>ABS(A9)</f>
+        <f>SQRT(ABS(A9))</f>
         <v>0</v>
       </c>
       <c r="CF9">
-        <f>SIGN(A9)</f>
+        <f>POWER(ABS(A9),2)</f>
         <v>0</v>
       </c>
       <c r="CG9">
-        <f>SQRT(ABS(A9))</f>
+        <f>CEILING(B9,1)</f>
         <v>0</v>
       </c>
       <c r="CH9">
-        <f>POWER(ABS(A9),2)</f>
+        <f>FLOOR(B9,1)</f>
         <v>0</v>
       </c>
       <c r="CI9">
-        <f>CEILING(B9,1)</f>
+        <f>LN(ABS(A9)+1)</f>
         <v>0</v>
       </c>
       <c r="CJ9">
-        <f>FLOOR(B9,1)</f>
+        <f>LOG(ABS(A9)+1,10)</f>
         <v>0</v>
       </c>
       <c r="CK9">
-        <f>LN(ABS(A9)+1)</f>
+        <f>LOG10(ABS(A9)+1)</f>
         <v>0</v>
       </c>
       <c r="CL9">
-        <f>LOG(ABS(A9)+1,10)</f>
+        <f>EXP(1)</f>
         <v>0</v>
       </c>
       <c r="CM9">
-        <f>LOG10(ABS(A9)+1)</f>
+        <f>SIN(B9)</f>
         <v>0</v>
       </c>
       <c r="CN9">
-        <f>EXP(1)</f>
+        <f>COS(B9)</f>
         <v>0</v>
       </c>
       <c r="CO9">
-        <f>SIN(B9)</f>
+        <f>TAN(B9)</f>
         <v>0</v>
       </c>
       <c r="CP9">
-        <f>COS(B9)</f>
+        <f>ASIN(B9/100)</f>
         <v>0</v>
       </c>
       <c r="CQ9">
-        <f>TAN(B9)</f>
+        <f>ACOS(B9/100)</f>
         <v>0</v>
       </c>
       <c r="CR9">
-        <f>ASIN(B9/100)</f>
+        <f>ATAN(B9)</f>
         <v>0</v>
       </c>
       <c r="CS9">
-        <f>ACOS(B9/100)</f>
+        <f>ATAN2(A9,B9)</f>
         <v>0</v>
       </c>
       <c r="CT9">
-        <f>ATAN(B9)</f>
+        <f>PI()</f>
         <v>0</v>
       </c>
       <c r="CU9">
-        <f>ATAN2(A9,B9)</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
       <c r="CV9">
-        <f>PI()</f>
+        <f>NOW()</f>
         <v>0</v>
       </c>
       <c r="CW9">
-        <f>TODAY()</f>
+        <f>DATE(2026,4,20)</f>
         <v>0</v>
       </c>
       <c r="CX9">
-        <f>NOW()</f>
+        <f>YEAR(G9)</f>
         <v>0</v>
       </c>
       <c r="CY9">
-        <f>DATE(2026,4,20)</f>
+        <f>MONTH(G9)</f>
         <v>0</v>
       </c>
       <c r="CZ9">
-        <f>YEAR(G9)</f>
+        <f>DAY(G9)</f>
         <v>0</v>
       </c>
       <c r="DA9">
-        <f>MONTH(G9)</f>
+        <f>WEEKDAY(G9)</f>
         <v>0</v>
       </c>
       <c r="DB9">
-        <f>DAY(G9)</f>
+        <f>EDATE(G9,3)</f>
         <v>0</v>
       </c>
       <c r="DC9">
-        <f>WEEKDAY(G9)</f>
+        <f>EOMONTH(G9,0)</f>
         <v>0</v>
       </c>
       <c r="DD9">
-        <f>EDATE(G9,3)</f>
+        <f>DATEDIF(DATE(2020,1,1),G9,"d")</f>
         <v>0</v>
       </c>
       <c r="DE9">
-        <f>EOMONTH(G9,0)</f>
+        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
         <v>0</v>
       </c>
       <c r="DF9">
-        <f>DATEDIF(DATE(2020,1,1),G9,"d")</f>
+        <f>WORKDAY(DATE(2026,1,1),10)</f>
         <v>0</v>
       </c>
       <c r="DG9">
-        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
+        <f>ISBLANK(H9)</f>
         <v>0</v>
       </c>
       <c r="DH9">
-        <f>WORKDAY(DATE(2026,1,1),10)</f>
+        <f>ISNUMBER(A9)</f>
         <v>0</v>
       </c>
       <c r="DI9">
-        <f>ISBLANK(H9)</f>
+        <f>ISTEXT(F9)</f>
         <v>0</v>
       </c>
       <c r="DJ9">
-        <f>ISNUMBER(A9)</f>
+        <f>ISLOGICAL(D9)</f>
         <v>0</v>
       </c>
       <c r="DK9">
-        <f>ISTEXT(F9)</f>
+        <f>ISNONTEXT(A9)</f>
         <v>0</v>
       </c>
       <c r="DL9">
-        <f>ISLOGICAL(D9)</f>
+        <f>ISERROR(1/0)</f>
         <v>0</v>
       </c>
       <c r="DM9">
-        <f>ISNONTEXT(A9)</f>
+        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="DN9">
-        <f>ISERROR(1/0)</f>
+        <f>ISREF(A9)</f>
         <v>0</v>
       </c>
       <c r="DO9">
-        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
+        <f>NA()</f>
         <v>0</v>
       </c>
       <c r="DP9">
-        <f>ISREF(A9)</f>
+        <f>TYPE(A9)</f>
         <v>0</v>
       </c>
       <c r="DQ9">
-        <f>NA()</f>
+        <f>PMT(0.05/12,360,-200000)</f>
         <v>0</v>
       </c>
       <c r="DR9">
-        <f>TYPE(A9)</f>
+        <f>PV(0.08/12,120,-500)</f>
         <v>0</v>
       </c>
       <c r="DS9">
-        <f>PMT(0.05/12,360,-200000)</f>
+        <f>FV(0.06/12,240,-200)</f>
         <v>0</v>
       </c>
       <c r="DT9">
-        <f>PV(0.08/12,120,-500)</f>
+        <f>NPV(0.1,A9,B9,C9)</f>
         <v>0</v>
       </c>
       <c r="DU9">
-        <f>FV(0.06/12,240,-200)</f>
-        <v>0</v>
-      </c>
-      <c r="DV9">
-        <f>NPV(0.1,A9,B9,C9)</f>
-        <v>0</v>
-      </c>
-      <c r="DW9">
         <f>RATE(120,-500,50000)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:127">
+    <row r="10" spans="1:125">
       <c r="A10">
         <v>999.0</v>
       </c>
@@ -5509,7 +5433,7 @@
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G10" s="1">
         <v>45400.0</v>
@@ -5682,319 +5606,311 @@
         <v>0</v>
       </c>
       <c r="AX10">
-        <f>_xlfn.MINIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
+        <f>VLOOKUP(E10,Lookup1!A:C,2,FALSE)</f>
         <v>0</v>
       </c>
       <c r="AY10">
-        <f>_xlfn.MAXIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
-        <v>0</v>
-      </c>
-      <c r="AZ10">
-        <f>VLOOKUP(E10,Lookup1!A:C,2,FALSE)</f>
+        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ10" cm="1">
+        <f t="array" ref="AZ10">_xlfn.XLOOKUP(E10,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
         <v>0</v>
       </c>
       <c r="BA10">
-        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BB10" cm="1">
-        <f t="array" ref="BB10">_xlfn.XLOOKUP(E10,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
+        <f>MATCH(E10,Lookup1!A:A,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BB10">
+        <f>_xlfn.XMATCH(E10,Lookup1!A:A,0)</f>
         <v>0</v>
       </c>
       <c r="BC10">
-        <f>MATCH(E10,Lookup1!A:A,0)</f>
+        <f>INDEX(Lookup1!B:B,MATCH(E10,Lookup1!A:A,0))</f>
         <v>0</v>
       </c>
       <c r="BD10">
-        <f>_xlfn.XMATCH(E10,Lookup1!A:A,0)</f>
+        <f>CHOOSE(2,"alpha","beta","gamma")</f>
         <v>0</v>
       </c>
       <c r="BE10">
-        <f>INDEX(Lookup1!B:B,MATCH(E10,Lookup1!A:A,0))</f>
+        <f>LEFT(F10,3)</f>
         <v>0</v>
       </c>
       <c r="BF10">
-        <f>CHOOSE(2,"alpha","beta","gamma")</f>
+        <f>RIGHT(F10,3)</f>
         <v>0</v>
       </c>
       <c r="BG10">
-        <f>LEFT(F10,3)</f>
+        <f>MID(F10,2,3)</f>
         <v>0</v>
       </c>
       <c r="BH10">
-        <f>RIGHT(F10,3)</f>
+        <f>LEN(F10)</f>
         <v>0</v>
       </c>
       <c r="BI10">
-        <f>MID(F10,2,3)</f>
+        <f>UPPER(F10)</f>
         <v>0</v>
       </c>
       <c r="BJ10">
-        <f>LEN(F10)</f>
+        <f>LOWER(F10)</f>
         <v>0</v>
       </c>
       <c r="BK10">
-        <f>UPPER(F10)</f>
+        <f>PROPER(F10)</f>
         <v>0</v>
       </c>
       <c r="BL10">
-        <f>LOWER(F10)</f>
+        <f>TRIM(F10)</f>
         <v>0</v>
       </c>
       <c r="BM10">
-        <f>PROPER(F10)</f>
+        <f>CLEAN(F10)</f>
         <v>0</v>
       </c>
       <c r="BN10">
-        <f>TRIM(F10)</f>
+        <f>_xlfn.CONCAT(E10,"-",F10)</f>
         <v>0</v>
       </c>
       <c r="BO10">
-        <f>CLEAN(F10)</f>
+        <f>CONCATENATE(E10,"-",F10)</f>
         <v>0</v>
       </c>
       <c r="BP10">
-        <f>_xlfn.CONCAT(E10,"-",F10)</f>
+        <f>_xlfn.TEXTJOIN("-",TRUE,E10,F10)</f>
         <v>0</v>
       </c>
       <c r="BQ10">
-        <f>CONCATENATE(E10,"-",F10)</f>
+        <f>IFERROR(FIND("l",F10),0)</f>
         <v>0</v>
       </c>
       <c r="BR10">
-        <f>_xlfn.TEXTJOIN("-",TRUE,E10,F10)</f>
+        <f>IFERROR(SEARCH("L",F10),0)</f>
         <v>0</v>
       </c>
       <c r="BS10">
-        <f>IFERROR(FIND("l",F10),0)</f>
+        <f>SUBSTITUTE(F10,"o","0")</f>
         <v>0</v>
       </c>
       <c r="BT10">
-        <f>IFERROR(SEARCH("L",F10),0)</f>
+        <f>REPLACE(F10,1,1,"X")</f>
         <v>0</v>
       </c>
       <c r="BU10">
-        <f>SUBSTITUTE(F10,"o","0")</f>
+        <f>TEXT(C10,"0.00")</f>
         <v>0</v>
       </c>
       <c r="BV10">
-        <f>REPLACE(F10,1,1,"X")</f>
+        <f>VALUE("123.45")</f>
         <v>0</v>
       </c>
       <c r="BW10">
-        <f>TEXT(C10,"0.00")</f>
+        <f>EXACT(F10,"hello")</f>
         <v>0</v>
       </c>
       <c r="BX10">
-        <f>VALUE("123.45")</f>
+        <f>ROUND(B10,1)</f>
         <v>0</v>
       </c>
       <c r="BY10">
-        <f>EXACT(F10,"hello")</f>
+        <f>ROUNDUP(B10,0)</f>
         <v>0</v>
       </c>
       <c r="BZ10">
-        <f>ROUND(B10,1)</f>
+        <f>ROUNDDOWN(B10,0)</f>
         <v>0</v>
       </c>
       <c r="CA10">
-        <f>ROUNDUP(B10,0)</f>
+        <f>INT(B10)</f>
         <v>0</v>
       </c>
       <c r="CB10">
-        <f>ROUNDDOWN(B10,0)</f>
+        <f>MOD(A10,3)</f>
         <v>0</v>
       </c>
       <c r="CC10">
-        <f>INT(B10)</f>
+        <f>ABS(A10)</f>
         <v>0</v>
       </c>
       <c r="CD10">
-        <f>MOD(A10,3)</f>
+        <f>SIGN(A10)</f>
         <v>0</v>
       </c>
       <c r="CE10">
-        <f>ABS(A10)</f>
+        <f>SQRT(ABS(A10))</f>
         <v>0</v>
       </c>
       <c r="CF10">
-        <f>SIGN(A10)</f>
+        <f>POWER(ABS(A10),2)</f>
         <v>0</v>
       </c>
       <c r="CG10">
-        <f>SQRT(ABS(A10))</f>
+        <f>CEILING(B10,1)</f>
         <v>0</v>
       </c>
       <c r="CH10">
-        <f>POWER(ABS(A10),2)</f>
+        <f>FLOOR(B10,1)</f>
         <v>0</v>
       </c>
       <c r="CI10">
-        <f>CEILING(B10,1)</f>
+        <f>LN(ABS(A10)+1)</f>
         <v>0</v>
       </c>
       <c r="CJ10">
-        <f>FLOOR(B10,1)</f>
+        <f>LOG(ABS(A10)+1,10)</f>
         <v>0</v>
       </c>
       <c r="CK10">
-        <f>LN(ABS(A10)+1)</f>
+        <f>LOG10(ABS(A10)+1)</f>
         <v>0</v>
       </c>
       <c r="CL10">
-        <f>LOG(ABS(A10)+1,10)</f>
+        <f>EXP(1)</f>
         <v>0</v>
       </c>
       <c r="CM10">
-        <f>LOG10(ABS(A10)+1)</f>
+        <f>SIN(B10)</f>
         <v>0</v>
       </c>
       <c r="CN10">
-        <f>EXP(1)</f>
+        <f>COS(B10)</f>
         <v>0</v>
       </c>
       <c r="CO10">
-        <f>SIN(B10)</f>
+        <f>TAN(B10)</f>
         <v>0</v>
       </c>
       <c r="CP10">
-        <f>COS(B10)</f>
+        <f>ASIN(B10/100)</f>
         <v>0</v>
       </c>
       <c r="CQ10">
-        <f>TAN(B10)</f>
+        <f>ACOS(B10/100)</f>
         <v>0</v>
       </c>
       <c r="CR10">
-        <f>ASIN(B10/100)</f>
+        <f>ATAN(B10)</f>
         <v>0</v>
       </c>
       <c r="CS10">
-        <f>ACOS(B10/100)</f>
+        <f>ATAN2(A10,B10)</f>
         <v>0</v>
       </c>
       <c r="CT10">
-        <f>ATAN(B10)</f>
+        <f>PI()</f>
         <v>0</v>
       </c>
       <c r="CU10">
-        <f>ATAN2(A10,B10)</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
       <c r="CV10">
-        <f>PI()</f>
+        <f>NOW()</f>
         <v>0</v>
       </c>
       <c r="CW10">
-        <f>TODAY()</f>
+        <f>DATE(2026,4,20)</f>
         <v>0</v>
       </c>
       <c r="CX10">
-        <f>NOW()</f>
+        <f>YEAR(G10)</f>
         <v>0</v>
       </c>
       <c r="CY10">
-        <f>DATE(2026,4,20)</f>
+        <f>MONTH(G10)</f>
         <v>0</v>
       </c>
       <c r="CZ10">
-        <f>YEAR(G10)</f>
+        <f>DAY(G10)</f>
         <v>0</v>
       </c>
       <c r="DA10">
-        <f>MONTH(G10)</f>
+        <f>WEEKDAY(G10)</f>
         <v>0</v>
       </c>
       <c r="DB10">
-        <f>DAY(G10)</f>
+        <f>EDATE(G10,3)</f>
         <v>0</v>
       </c>
       <c r="DC10">
-        <f>WEEKDAY(G10)</f>
+        <f>EOMONTH(G10,0)</f>
         <v>0</v>
       </c>
       <c r="DD10">
-        <f>EDATE(G10,3)</f>
+        <f>DATEDIF(DATE(2020,1,1),G10,"d")</f>
         <v>0</v>
       </c>
       <c r="DE10">
-        <f>EOMONTH(G10,0)</f>
+        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
         <v>0</v>
       </c>
       <c r="DF10">
-        <f>DATEDIF(DATE(2020,1,1),G10,"d")</f>
+        <f>WORKDAY(DATE(2026,1,1),10)</f>
         <v>0</v>
       </c>
       <c r="DG10">
-        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
+        <f>ISBLANK(H10)</f>
         <v>0</v>
       </c>
       <c r="DH10">
-        <f>WORKDAY(DATE(2026,1,1),10)</f>
+        <f>ISNUMBER(A10)</f>
         <v>0</v>
       </c>
       <c r="DI10">
-        <f>ISBLANK(H10)</f>
+        <f>ISTEXT(F10)</f>
         <v>0</v>
       </c>
       <c r="DJ10">
-        <f>ISNUMBER(A10)</f>
+        <f>ISLOGICAL(D10)</f>
         <v>0</v>
       </c>
       <c r="DK10">
-        <f>ISTEXT(F10)</f>
+        <f>ISNONTEXT(A10)</f>
         <v>0</v>
       </c>
       <c r="DL10">
-        <f>ISLOGICAL(D10)</f>
+        <f>ISERROR(1/0)</f>
         <v>0</v>
       </c>
       <c r="DM10">
-        <f>ISNONTEXT(A10)</f>
+        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="DN10">
-        <f>ISERROR(1/0)</f>
+        <f>ISREF(A10)</f>
         <v>0</v>
       </c>
       <c r="DO10">
-        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
+        <f>NA()</f>
         <v>0</v>
       </c>
       <c r="DP10">
-        <f>ISREF(A10)</f>
+        <f>TYPE(A10)</f>
         <v>0</v>
       </c>
       <c r="DQ10">
-        <f>NA()</f>
+        <f>PMT(0.05/12,360,-200000)</f>
         <v>0</v>
       </c>
       <c r="DR10">
-        <f>TYPE(A10)</f>
+        <f>PV(0.08/12,120,-500)</f>
         <v>0</v>
       </c>
       <c r="DS10">
-        <f>PMT(0.05/12,360,-200000)</f>
+        <f>FV(0.06/12,240,-200)</f>
         <v>0</v>
       </c>
       <c r="DT10">
-        <f>PV(0.08/12,120,-500)</f>
+        <f>NPV(0.1,A10,B10,C10)</f>
         <v>0</v>
       </c>
       <c r="DU10">
-        <f>FV(0.06/12,240,-200)</f>
-        <v>0</v>
-      </c>
-      <c r="DV10">
-        <f>NPV(0.1,A10,B10,C10)</f>
-        <v>0</v>
-      </c>
-      <c r="DW10">
         <f>RATE(120,-500,50000)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:127">
+    <row r="11" spans="1:125">
       <c r="A11">
         <v>42.0</v>
       </c>
@@ -6011,7 +5927,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G11" s="1">
         <v>45500.0</v>
@@ -6181,314 +6097,306 @@
         <v>0</v>
       </c>
       <c r="AX11">
-        <f>_xlfn.MINIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
+        <f>VLOOKUP(E11,Lookup1!A:C,2,FALSE)</f>
         <v>0</v>
       </c>
       <c r="AY11">
-        <f>_xlfn.MAXIFS(AggSource!B:B,AggSource!A:A,"EMEA",AggSource!C:C,"Sales")</f>
-        <v>0</v>
-      </c>
-      <c r="AZ11">
-        <f>VLOOKUP(E11,Lookup1!A:C,2,FALSE)</f>
+        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="AZ11" cm="1">
+        <f t="array" ref="AZ11">_xlfn.XLOOKUP(E11,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
         <v>0</v>
       </c>
       <c r="BA11">
-        <f>HLOOKUP("Q2",HLookup!A1:D3,2,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BB11" cm="1">
-        <f t="array" ref="BB11">_xlfn.XLOOKUP(E11,Lookup1!A:A,Lookup1!B:B,"N/F")</f>
+        <f>MATCH(E11,Lookup1!A:A,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BB11">
+        <f>_xlfn.XMATCH(E11,Lookup1!A:A,0)</f>
         <v>0</v>
       </c>
       <c r="BC11">
-        <f>MATCH(E11,Lookup1!A:A,0)</f>
+        <f>INDEX(Lookup1!B:B,MATCH(E11,Lookup1!A:A,0))</f>
         <v>0</v>
       </c>
       <c r="BD11">
-        <f>_xlfn.XMATCH(E11,Lookup1!A:A,0)</f>
+        <f>CHOOSE(2,"alpha","beta","gamma")</f>
         <v>0</v>
       </c>
       <c r="BE11">
-        <f>INDEX(Lookup1!B:B,MATCH(E11,Lookup1!A:A,0))</f>
+        <f>LEFT(F11,3)</f>
         <v>0</v>
       </c>
       <c r="BF11">
-        <f>CHOOSE(2,"alpha","beta","gamma")</f>
+        <f>RIGHT(F11,3)</f>
         <v>0</v>
       </c>
       <c r="BG11">
-        <f>LEFT(F11,3)</f>
+        <f>MID(F11,2,3)</f>
         <v>0</v>
       </c>
       <c r="BH11">
-        <f>RIGHT(F11,3)</f>
+        <f>LEN(F11)</f>
         <v>0</v>
       </c>
       <c r="BI11">
-        <f>MID(F11,2,3)</f>
+        <f>UPPER(F11)</f>
         <v>0</v>
       </c>
       <c r="BJ11">
-        <f>LEN(F11)</f>
+        <f>LOWER(F11)</f>
         <v>0</v>
       </c>
       <c r="BK11">
-        <f>UPPER(F11)</f>
+        <f>PROPER(F11)</f>
         <v>0</v>
       </c>
       <c r="BL11">
-        <f>LOWER(F11)</f>
+        <f>TRIM(F11)</f>
         <v>0</v>
       </c>
       <c r="BM11">
-        <f>PROPER(F11)</f>
+        <f>CLEAN(F11)</f>
         <v>0</v>
       </c>
       <c r="BN11">
-        <f>TRIM(F11)</f>
+        <f>_xlfn.CONCAT(E11,"-",F11)</f>
         <v>0</v>
       </c>
       <c r="BO11">
-        <f>CLEAN(F11)</f>
+        <f>CONCATENATE(E11,"-",F11)</f>
         <v>0</v>
       </c>
       <c r="BP11">
-        <f>_xlfn.CONCAT(E11,"-",F11)</f>
+        <f>_xlfn.TEXTJOIN("-",TRUE,E11,F11)</f>
         <v>0</v>
       </c>
       <c r="BQ11">
-        <f>CONCATENATE(E11,"-",F11)</f>
+        <f>IFERROR(FIND("l",F11),0)</f>
         <v>0</v>
       </c>
       <c r="BR11">
-        <f>_xlfn.TEXTJOIN("-",TRUE,E11,F11)</f>
+        <f>IFERROR(SEARCH("L",F11),0)</f>
         <v>0</v>
       </c>
       <c r="BS11">
-        <f>IFERROR(FIND("l",F11),0)</f>
+        <f>SUBSTITUTE(F11,"o","0")</f>
         <v>0</v>
       </c>
       <c r="BT11">
-        <f>IFERROR(SEARCH("L",F11),0)</f>
+        <f>REPLACE(F11,1,1,"X")</f>
         <v>0</v>
       </c>
       <c r="BU11">
-        <f>SUBSTITUTE(F11,"o","0")</f>
+        <f>TEXT(C11,"0.00")</f>
         <v>0</v>
       </c>
       <c r="BV11">
-        <f>REPLACE(F11,1,1,"X")</f>
+        <f>VALUE("123.45")</f>
         <v>0</v>
       </c>
       <c r="BW11">
-        <f>TEXT(C11,"0.00")</f>
+        <f>EXACT(F11,"hello")</f>
         <v>0</v>
       </c>
       <c r="BX11">
-        <f>VALUE("123.45")</f>
+        <f>ROUND(B11,1)</f>
         <v>0</v>
       </c>
       <c r="BY11">
-        <f>EXACT(F11,"hello")</f>
+        <f>ROUNDUP(B11,0)</f>
         <v>0</v>
       </c>
       <c r="BZ11">
-        <f>ROUND(B11,1)</f>
+        <f>ROUNDDOWN(B11,0)</f>
         <v>0</v>
       </c>
       <c r="CA11">
-        <f>ROUNDUP(B11,0)</f>
+        <f>INT(B11)</f>
         <v>0</v>
       </c>
       <c r="CB11">
-        <f>ROUNDDOWN(B11,0)</f>
+        <f>MOD(A11,3)</f>
         <v>0</v>
       </c>
       <c r="CC11">
-        <f>INT(B11)</f>
+        <f>ABS(A11)</f>
         <v>0</v>
       </c>
       <c r="CD11">
-        <f>MOD(A11,3)</f>
+        <f>SIGN(A11)</f>
         <v>0</v>
       </c>
       <c r="CE11">
-        <f>ABS(A11)</f>
+        <f>SQRT(ABS(A11))</f>
         <v>0</v>
       </c>
       <c r="CF11">
-        <f>SIGN(A11)</f>
+        <f>POWER(ABS(A11),2)</f>
         <v>0</v>
       </c>
       <c r="CG11">
-        <f>SQRT(ABS(A11))</f>
+        <f>CEILING(B11,1)</f>
         <v>0</v>
       </c>
       <c r="CH11">
-        <f>POWER(ABS(A11),2)</f>
+        <f>FLOOR(B11,1)</f>
         <v>0</v>
       </c>
       <c r="CI11">
-        <f>CEILING(B11,1)</f>
+        <f>LN(ABS(A11)+1)</f>
         <v>0</v>
       </c>
       <c r="CJ11">
-        <f>FLOOR(B11,1)</f>
+        <f>LOG(ABS(A11)+1,10)</f>
         <v>0</v>
       </c>
       <c r="CK11">
-        <f>LN(ABS(A11)+1)</f>
+        <f>LOG10(ABS(A11)+1)</f>
         <v>0</v>
       </c>
       <c r="CL11">
-        <f>LOG(ABS(A11)+1,10)</f>
+        <f>EXP(1)</f>
         <v>0</v>
       </c>
       <c r="CM11">
-        <f>LOG10(ABS(A11)+1)</f>
+        <f>SIN(B11)</f>
         <v>0</v>
       </c>
       <c r="CN11">
-        <f>EXP(1)</f>
+        <f>COS(B11)</f>
         <v>0</v>
       </c>
       <c r="CO11">
-        <f>SIN(B11)</f>
+        <f>TAN(B11)</f>
         <v>0</v>
       </c>
       <c r="CP11">
-        <f>COS(B11)</f>
+        <f>ASIN(B11/100)</f>
         <v>0</v>
       </c>
       <c r="CQ11">
-        <f>TAN(B11)</f>
+        <f>ACOS(B11/100)</f>
         <v>0</v>
       </c>
       <c r="CR11">
-        <f>ASIN(B11/100)</f>
+        <f>ATAN(B11)</f>
         <v>0</v>
       </c>
       <c r="CS11">
-        <f>ACOS(B11/100)</f>
+        <f>ATAN2(A11,B11)</f>
         <v>0</v>
       </c>
       <c r="CT11">
-        <f>ATAN(B11)</f>
+        <f>PI()</f>
         <v>0</v>
       </c>
       <c r="CU11">
-        <f>ATAN2(A11,B11)</f>
+        <f>TODAY()</f>
         <v>0</v>
       </c>
       <c r="CV11">
-        <f>PI()</f>
+        <f>NOW()</f>
         <v>0</v>
       </c>
       <c r="CW11">
-        <f>TODAY()</f>
+        <f>DATE(2026,4,20)</f>
         <v>0</v>
       </c>
       <c r="CX11">
-        <f>NOW()</f>
+        <f>YEAR(G11)</f>
         <v>0</v>
       </c>
       <c r="CY11">
-        <f>DATE(2026,4,20)</f>
+        <f>MONTH(G11)</f>
         <v>0</v>
       </c>
       <c r="CZ11">
-        <f>YEAR(G11)</f>
+        <f>DAY(G11)</f>
         <v>0</v>
       </c>
       <c r="DA11">
-        <f>MONTH(G11)</f>
+        <f>WEEKDAY(G11)</f>
         <v>0</v>
       </c>
       <c r="DB11">
-        <f>DAY(G11)</f>
+        <f>EDATE(G11,3)</f>
         <v>0</v>
       </c>
       <c r="DC11">
-        <f>WEEKDAY(G11)</f>
+        <f>EOMONTH(G11,0)</f>
         <v>0</v>
       </c>
       <c r="DD11">
-        <f>EDATE(G11,3)</f>
+        <f>DATEDIF(DATE(2020,1,1),G11,"d")</f>
         <v>0</v>
       </c>
       <c r="DE11">
-        <f>EOMONTH(G11,0)</f>
+        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
         <v>0</v>
       </c>
       <c r="DF11">
-        <f>DATEDIF(DATE(2020,1,1),G11,"d")</f>
+        <f>WORKDAY(DATE(2026,1,1),10)</f>
         <v>0</v>
       </c>
       <c r="DG11">
-        <f>NETWORKDAYS(DATE(2026,1,1),DATE(2026,1,31))</f>
+        <f>ISBLANK(H11)</f>
         <v>0</v>
       </c>
       <c r="DH11">
-        <f>WORKDAY(DATE(2026,1,1),10)</f>
+        <f>ISNUMBER(A11)</f>
         <v>0</v>
       </c>
       <c r="DI11">
-        <f>ISBLANK(H11)</f>
+        <f>ISTEXT(F11)</f>
         <v>0</v>
       </c>
       <c r="DJ11">
-        <f>ISNUMBER(A11)</f>
+        <f>ISLOGICAL(D11)</f>
         <v>0</v>
       </c>
       <c r="DK11">
-        <f>ISTEXT(F11)</f>
+        <f>ISNONTEXT(A11)</f>
         <v>0</v>
       </c>
       <c r="DL11">
-        <f>ISLOGICAL(D11)</f>
+        <f>ISERROR(1/0)</f>
         <v>0</v>
       </c>
       <c r="DM11">
-        <f>ISNONTEXT(A11)</f>
+        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
         <v>0</v>
       </c>
       <c r="DN11">
-        <f>ISERROR(1/0)</f>
+        <f>ISREF(A11)</f>
         <v>0</v>
       </c>
       <c r="DO11">
-        <f>ISNA(VLOOKUP("ZZZ",Lookup1!A:C,2,FALSE))</f>
+        <f>NA()</f>
         <v>0</v>
       </c>
       <c r="DP11">
-        <f>ISREF(A11)</f>
+        <f>TYPE(A11)</f>
         <v>0</v>
       </c>
       <c r="DQ11">
-        <f>NA()</f>
+        <f>PMT(0.05/12,360,-200000)</f>
         <v>0</v>
       </c>
       <c r="DR11">
-        <f>TYPE(A11)</f>
+        <f>PV(0.08/12,120,-500)</f>
         <v>0</v>
       </c>
       <c r="DS11">
-        <f>PMT(0.05/12,360,-200000)</f>
+        <f>FV(0.06/12,240,-200)</f>
         <v>0</v>
       </c>
       <c r="DT11">
-        <f>PV(0.08/12,120,-500)</f>
+        <f>NPV(0.1,A11,B11,C11)</f>
         <v>0</v>
       </c>
       <c r="DU11">
-        <f>FV(0.06/12,240,-200)</f>
-        <v>0</v>
-      </c>
-      <c r="DV11">
-        <f>NPV(0.1,A11,B11,C11)</f>
-        <v>0</v>
-      </c>
-      <c r="DW11">
         <f>RATE(120,-500,50000)</f>
         <v>0</v>
       </c>

</xml_diff>